<commit_message>
Update Historical_Starting_Pitchers with today's starters (2026-03-30)
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/data/mlb/Historical_Starting_Pitchers.xlsx
+++ b/backend/data/mlb/Historical_Starting_Pitchers.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="568" uniqueCount="286">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="574" uniqueCount="287">
   <si>
     <t>Baseball_Savant_Name</t>
   </si>
@@ -25,6 +25,78 @@
     <t>Handedness</t>
   </si>
   <si>
+    <t>Bryce Elder</t>
+  </si>
+  <si>
+    <t>Chris Bassitt</t>
+  </si>
+  <si>
+    <t>Chris Paddack</t>
+  </si>
+  <si>
+    <t>Clay Holmes</t>
+  </si>
+  <si>
+    <t>Davis Martin</t>
+  </si>
+  <si>
+    <t>Edward Cabrera</t>
+  </si>
+  <si>
+    <t>Jack Leiter</t>
+  </si>
+  <si>
+    <t>Justin Verlander</t>
+  </si>
+  <si>
+    <t>Kris Bubic</t>
+  </si>
+  <si>
+    <t>Kyle Harrison</t>
+  </si>
+  <si>
+    <t>Landen Roupp</t>
+  </si>
+  <si>
+    <t>Luis Castillo</t>
+  </si>
+  <si>
+    <t>Michael Soroka</t>
+  </si>
+  <si>
+    <t>Nick Martinez</t>
+  </si>
+  <si>
+    <t>Ranger Suárez</t>
+  </si>
+  <si>
+    <t>Ryan Weathers</t>
+  </si>
+  <si>
+    <t>Simeon Woods Richardson</t>
+  </si>
+  <si>
+    <t>Taijuan Walker</t>
+  </si>
+  <si>
+    <t>Walker Buehler</t>
+  </si>
+  <si>
+    <t>Roki Sasaki</t>
+  </si>
+  <si>
+    <t>Tomoyuki Sugano</t>
+  </si>
+  <si>
+    <t>Jacob Lopez</t>
+  </si>
+  <si>
+    <t>Braxton Ashcraft</t>
+  </si>
+  <si>
+    <t>Chase Burns</t>
+  </si>
+  <si>
     <t>Cristopher Sánchez</t>
   </si>
   <si>
@@ -142,9 +214,6 @@
     <t>Emmet Sheehan</t>
   </si>
   <si>
-    <t>Jack Leiter</t>
-  </si>
-  <si>
     <t>Jameson Taillon</t>
   </si>
   <si>
@@ -160,15 +229,9 @@
     <t>Mitchell Parker</t>
   </si>
   <si>
-    <t>Ranger Suárez</t>
-  </si>
-  <si>
     <t>Sean Burke</t>
   </si>
   <si>
-    <t>Simeon Woods Richardson</t>
-  </si>
-  <si>
     <t>Spencer Strider</t>
   </si>
   <si>
@@ -181,9 +244,6 @@
     <t>Jason Alexander</t>
   </si>
   <si>
-    <t>Braxton Ashcraft</t>
-  </si>
-  <si>
     <t>Kai-Wei Teng</t>
   </si>
   <si>
@@ -208,9 +268,6 @@
     <t>Colin Rea</t>
   </si>
   <si>
-    <t>Davis Martin</t>
-  </si>
-  <si>
     <t>Drew Rasmussen</t>
   </si>
   <si>
@@ -223,9 +280,6 @@
     <t>Hunter Greene</t>
   </si>
   <si>
-    <t>Luis Castillo</t>
-  </si>
-  <si>
     <t>Luis Severino</t>
   </si>
   <si>
@@ -247,15 +301,9 @@
     <t>Sonny Gray</t>
   </si>
   <si>
-    <t>Taijuan Walker</t>
-  </si>
-  <si>
     <t>Tanner Gordon</t>
   </si>
   <si>
-    <t>Tomoyuki Sugano</t>
-  </si>
-  <si>
     <t>Jacob Misiorowski</t>
   </si>
   <si>
@@ -289,9 +337,6 @@
     <t>Bryce Miller</t>
   </si>
   <si>
-    <t>Chris Bassitt</t>
-  </si>
-  <si>
     <t>Hunter Brown</t>
   </si>
   <si>
@@ -310,9 +355,6 @@
     <t>Joe Ryan</t>
   </si>
   <si>
-    <t>Justin Verlander</t>
-  </si>
-  <si>
     <t>Lucas Giolito</t>
   </si>
   <si>
@@ -433,15 +475,9 @@
     <t>Adrian Houser</t>
   </si>
   <si>
-    <t>Bryce Elder</t>
-  </si>
-  <si>
     <t>Cade Povich</t>
   </si>
   <si>
-    <t>Clay Holmes</t>
-  </si>
-  <si>
     <t>Dustin May</t>
   </si>
   <si>
@@ -532,15 +568,9 @@
     <t>Kyle Hart</t>
   </si>
   <si>
-    <t>Edward Cabrera</t>
-  </si>
-  <si>
     <t>Spencer Arrighetti</t>
   </si>
   <si>
-    <t>Chris Paddack</t>
-  </si>
-  <si>
     <t>Seth Lugo</t>
   </si>
   <si>
@@ -568,9 +598,6 @@
     <t>Ryan Gusto</t>
   </si>
   <si>
-    <t>Nick Martinez</t>
-  </si>
-  <si>
     <t>Osvaldo Bido</t>
   </si>
   <si>
@@ -583,9 +610,6 @@
     <t>Robert Gasser</t>
   </si>
   <si>
-    <t>Jacob Lopez</t>
-  </si>
-  <si>
     <t>Janson Junk</t>
   </si>
   <si>
@@ -607,15 +631,9 @@
     <t>Jack Perkins</t>
   </si>
   <si>
-    <t>Landen Roupp</t>
-  </si>
-  <si>
     <t>Austin Gomber</t>
   </si>
   <si>
-    <t>Walker Buehler</t>
-  </si>
-  <si>
     <t>Chad Patrick</t>
   </si>
   <si>
@@ -634,9 +652,6 @@
     <t>Bailey Falter</t>
   </si>
   <si>
-    <t>Michael Soroka</t>
-  </si>
-  <si>
     <t>Travis Adams</t>
   </si>
   <si>
@@ -667,9 +682,6 @@
     <t>Zach Eflin</t>
   </si>
   <si>
-    <t>Chase Burns</t>
-  </si>
-  <si>
     <t>Troy Melton</t>
   </si>
   <si>
@@ -682,9 +694,6 @@
     <t>Grant Holmes</t>
   </si>
   <si>
-    <t>Kris Bubic</t>
-  </si>
-  <si>
     <t>Davis Daniel</t>
   </si>
   <si>
@@ -760,9 +769,6 @@
     <t>Griffin Canning</t>
   </si>
   <si>
-    <t>Kyle Harrison</t>
-  </si>
-  <si>
     <t>Mitch Spence</t>
   </si>
   <si>
@@ -790,9 +796,6 @@
     <t>Caleb Boushley</t>
   </si>
   <si>
-    <t>Ryan Weathers</t>
-  </si>
-  <si>
     <t>Joe Ross</t>
   </si>
   <si>
@@ -868,10 +871,10 @@
     <t>Nathan Wiles</t>
   </si>
   <si>
+    <t>RHP</t>
+  </si>
+  <si>
     <t>LHP</t>
-  </si>
-  <si>
-    <t>RHP</t>
   </si>
 </sst>
 </file>
@@ -1229,7 +1232,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C284"/>
+  <dimension ref="A1:C289"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:3">
@@ -1248,10 +1251,10 @@
         <v>3</v>
       </c>
       <c r="B2">
-        <v>650911</v>
+        <v>693821</v>
       </c>
       <c r="C2" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
     </row>
     <row r="3" spans="1:3">
@@ -1259,7 +1262,7 @@
         <v>4</v>
       </c>
       <c r="B3">
-        <v>642547</v>
+        <v>605135</v>
       </c>
       <c r="C3" t="s">
         <v>285</v>
@@ -1270,7 +1273,7 @@
         <v>5</v>
       </c>
       <c r="B4">
-        <v>669923</v>
+        <v>663978</v>
       </c>
       <c r="C4" t="s">
         <v>285</v>
@@ -1281,29 +1284,23 @@
         <v>6</v>
       </c>
       <c r="B5">
-        <v>672456</v>
+        <v>605280</v>
       </c>
       <c r="C5" t="s">
         <v>285</v>
       </c>
     </row>
     <row r="6" spans="1:3">
-      <c r="A6" t="s">
-        <v>7</v>
-      </c>
-      <c r="B6">
-        <v>592332</v>
-      </c>
       <c r="C6" t="s">
         <v>285</v>
       </c>
     </row>
     <row r="7" spans="1:3">
       <c r="A7" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B7">
-        <v>661563</v>
+        <v>663436</v>
       </c>
       <c r="C7" t="s">
         <v>285</v>
@@ -1311,43 +1308,40 @@
     </row>
     <row r="8" spans="1:3">
       <c r="A8" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B8">
-        <v>571510</v>
+        <v>665795</v>
       </c>
       <c r="C8" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
     </row>
     <row r="9" spans="1:3">
-      <c r="A9" t="s">
-        <v>10</v>
-      </c>
       <c r="B9">
-        <v>660271</v>
+        <v>656492</v>
       </c>
       <c r="C9" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="10" spans="1:3">
       <c r="A10" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="B10">
-        <v>671096</v>
+        <v>683004</v>
       </c>
       <c r="C10" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
     </row>
     <row r="11" spans="1:3">
       <c r="A11" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="B11">
-        <v>702674</v>
+        <v>434378</v>
       </c>
       <c r="C11" t="s">
         <v>285</v>
@@ -1355,32 +1349,32 @@
     </row>
     <row r="12" spans="1:3">
       <c r="A12" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="B12">
-        <v>663554</v>
+        <v>663460</v>
       </c>
       <c r="C12" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="13" spans="1:3">
       <c r="A13" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B13">
-        <v>519242</v>
+        <v>690986</v>
       </c>
       <c r="C13" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
     </row>
     <row r="14" spans="1:3">
       <c r="A14" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="B14">
-        <v>665152</v>
+        <v>689017</v>
       </c>
       <c r="C14" t="s">
         <v>285</v>
@@ -1388,21 +1382,21 @@
     </row>
     <row r="15" spans="1:3">
       <c r="A15" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="B15">
-        <v>593958</v>
+        <v>622491</v>
       </c>
       <c r="C15" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
     </row>
     <row r="16" spans="1:3">
       <c r="A16" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B16">
-        <v>691587</v>
+        <v>647336</v>
       </c>
       <c r="C16" t="s">
         <v>285</v>
@@ -1410,10 +1404,10 @@
     </row>
     <row r="17" spans="1:3">
       <c r="A17" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
       <c r="B17">
-        <v>663623</v>
+        <v>607259</v>
       </c>
       <c r="C17" t="s">
         <v>285</v>
@@ -1421,32 +1415,32 @@
     </row>
     <row r="18" spans="1:3">
       <c r="A18" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="B18">
-        <v>605488</v>
+        <v>624133</v>
       </c>
       <c r="C18" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
     </row>
     <row r="19" spans="1:3">
       <c r="A19" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="B19">
-        <v>676282</v>
+        <v>677960</v>
       </c>
       <c r="C19" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
     </row>
     <row r="20" spans="1:3">
       <c r="A20" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="B20">
-        <v>621244</v>
+        <v>680573</v>
       </c>
       <c r="C20" t="s">
         <v>285</v>
@@ -1454,32 +1448,32 @@
     </row>
     <row r="21" spans="1:3">
       <c r="A21" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="B21">
-        <v>660761</v>
+        <v>592836</v>
       </c>
       <c r="C21" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
     </row>
     <row r="22" spans="1:3">
       <c r="A22" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="B22">
-        <v>607536</v>
+        <v>621111</v>
       </c>
       <c r="C22" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
     </row>
     <row r="23" spans="1:3">
       <c r="A23" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B23">
-        <v>669302</v>
+        <v>808963</v>
       </c>
       <c r="C23" t="s">
         <v>285</v>
@@ -1487,32 +1481,32 @@
     </row>
     <row r="24" spans="1:3">
       <c r="A24" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="B24">
-        <v>669022</v>
+        <v>608372</v>
       </c>
       <c r="C24" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
     </row>
     <row r="25" spans="1:3">
       <c r="A25" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B25">
-        <v>518876</v>
+        <v>682052</v>
       </c>
       <c r="C25" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="26" spans="1:3">
       <c r="A26" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="B26">
-        <v>650633</v>
+        <v>677952</v>
       </c>
       <c r="C26" t="s">
         <v>285</v>
@@ -1520,65 +1514,56 @@
     </row>
     <row r="27" spans="1:3">
       <c r="A27" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="B27">
-        <v>700241</v>
+        <v>695505</v>
       </c>
       <c r="C27" t="s">
         <v>285</v>
       </c>
     </row>
     <row r="28" spans="1:3">
-      <c r="A28" t="s">
-        <v>29</v>
-      </c>
       <c r="B28">
-        <v>608379</v>
+        <v>696270</v>
       </c>
       <c r="C28" t="s">
         <v>285</v>
       </c>
     </row>
     <row r="29" spans="1:3">
-      <c r="A29" t="s">
-        <v>30</v>
-      </c>
       <c r="B29">
-        <v>694973</v>
+        <v>681517</v>
       </c>
       <c r="C29" t="s">
         <v>285</v>
       </c>
     </row>
     <row r="30" spans="1:3">
-      <c r="A30" t="s">
-        <v>31</v>
-      </c>
       <c r="B30">
-        <v>686752</v>
+        <v>800048</v>
       </c>
       <c r="C30" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="31" spans="1:3">
       <c r="A31" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="B31">
-        <v>640455</v>
+        <v>650911</v>
       </c>
       <c r="C31" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
     </row>
     <row r="32" spans="1:3">
       <c r="A32" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="B32">
-        <v>663941</v>
+        <v>642547</v>
       </c>
       <c r="C32" t="s">
         <v>285</v>
@@ -1586,10 +1571,10 @@
     </row>
     <row r="33" spans="1:3">
       <c r="A33" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="B33">
-        <v>805673</v>
+        <v>669923</v>
       </c>
       <c r="C33" t="s">
         <v>285</v>
@@ -1597,10 +1582,10 @@
     </row>
     <row r="34" spans="1:3">
       <c r="A34" t="s">
-        <v>35</v>
+        <v>30</v>
       </c>
       <c r="B34">
-        <v>681343</v>
+        <v>672456</v>
       </c>
       <c r="C34" t="s">
         <v>285</v>
@@ -1608,10 +1593,10 @@
     </row>
     <row r="35" spans="1:3">
       <c r="A35" t="s">
-        <v>36</v>
+        <v>31</v>
       </c>
       <c r="B35">
-        <v>690990</v>
+        <v>592332</v>
       </c>
       <c r="C35" t="s">
         <v>285</v>
@@ -1619,10 +1604,10 @@
     </row>
     <row r="36" spans="1:3">
       <c r="A36" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="B36">
-        <v>693645</v>
+        <v>661563</v>
       </c>
       <c r="C36" t="s">
         <v>285</v>
@@ -1630,21 +1615,21 @@
     </row>
     <row r="37" spans="1:3">
       <c r="A37" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="B37">
-        <v>813349</v>
+        <v>571510</v>
       </c>
       <c r="C37" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
     </row>
     <row r="38" spans="1:3">
       <c r="A38" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="B38">
-        <v>805123</v>
+        <v>660271</v>
       </c>
       <c r="C38" t="s">
         <v>285</v>
@@ -1652,21 +1637,21 @@
     </row>
     <row r="39" spans="1:3">
       <c r="A39" t="s">
-        <v>40</v>
+        <v>35</v>
       </c>
       <c r="B39">
-        <v>607074</v>
+        <v>671096</v>
       </c>
       <c r="C39" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
     </row>
     <row r="40" spans="1:3">
       <c r="A40" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="B40">
-        <v>686218</v>
+        <v>702674</v>
       </c>
       <c r="C40" t="s">
         <v>285</v>
@@ -1674,10 +1659,10 @@
     </row>
     <row r="41" spans="1:3">
       <c r="A41" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="B41">
-        <v>683004</v>
+        <v>663554</v>
       </c>
       <c r="C41" t="s">
         <v>285</v>
@@ -1685,21 +1670,21 @@
     </row>
     <row r="42" spans="1:3">
       <c r="A42" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="B42">
-        <v>592791</v>
+        <v>519242</v>
       </c>
       <c r="C42" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="43" spans="1:3">
       <c r="A43" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="B43">
-        <v>671212</v>
+        <v>665152</v>
       </c>
       <c r="C43" t="s">
         <v>285</v>
@@ -1707,65 +1692,65 @@
     </row>
     <row r="44" spans="1:3">
       <c r="A44" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="B44">
-        <v>680694</v>
+        <v>593958</v>
       </c>
       <c r="C44" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="45" spans="1:3">
       <c r="A45" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="B45">
-        <v>669461</v>
+        <v>691587</v>
       </c>
       <c r="C45" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
     </row>
     <row r="46" spans="1:3">
       <c r="A46" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="B46">
-        <v>680730</v>
+        <v>663623</v>
       </c>
       <c r="C46" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
     </row>
     <row r="47" spans="1:3">
       <c r="A47" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="B47">
-        <v>624133</v>
+        <v>605488</v>
       </c>
       <c r="C47" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
     </row>
     <row r="48" spans="1:3">
       <c r="A48" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="B48">
-        <v>680732</v>
+        <v>676282</v>
       </c>
       <c r="C48" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="49" spans="1:3">
       <c r="A49" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="B49">
-        <v>680573</v>
+        <v>621244</v>
       </c>
       <c r="C49" t="s">
         <v>285</v>
@@ -1773,32 +1758,32 @@
     </row>
     <row r="50" spans="1:3">
       <c r="A50" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="B50">
-        <v>675911</v>
+        <v>660761</v>
       </c>
       <c r="C50" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="51" spans="1:3">
       <c r="A51" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="B51">
-        <v>668678</v>
+        <v>607536</v>
       </c>
       <c r="C51" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="52" spans="1:3">
       <c r="A52" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="B52">
-        <v>641793</v>
+        <v>669302</v>
       </c>
       <c r="C52" t="s">
         <v>285</v>
@@ -1806,21 +1791,21 @@
     </row>
     <row r="53" spans="1:3">
       <c r="A53" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="B53">
-        <v>669920</v>
+        <v>669022</v>
       </c>
       <c r="C53" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="54" spans="1:3">
       <c r="A54" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="B54">
-        <v>677952</v>
+        <v>518876</v>
       </c>
       <c r="C54" t="s">
         <v>285</v>
@@ -1828,10 +1813,10 @@
     </row>
     <row r="55" spans="1:3">
       <c r="A55" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="B55">
-        <v>678906</v>
+        <v>650633</v>
       </c>
       <c r="C55" t="s">
         <v>285</v>
@@ -1839,10 +1824,10 @@
     </row>
     <row r="56" spans="1:3">
       <c r="A56" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="B56">
-        <v>702056</v>
+        <v>700241</v>
       </c>
       <c r="C56" t="s">
         <v>285</v>
@@ -1850,10 +1835,10 @@
     </row>
     <row r="57" spans="1:3">
       <c r="A57" t="s">
-        <v>58</v>
+        <v>53</v>
       </c>
       <c r="B57">
-        <v>800049</v>
+        <v>608379</v>
       </c>
       <c r="C57" t="s">
         <v>285</v>
@@ -1861,10 +1846,10 @@
     </row>
     <row r="58" spans="1:3">
       <c r="A58" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="B58">
-        <v>641927</v>
+        <v>694973</v>
       </c>
       <c r="C58" t="s">
         <v>285</v>
@@ -1872,10 +1857,10 @@
     </row>
     <row r="59" spans="1:3">
       <c r="A59" t="s">
-        <v>60</v>
+        <v>55</v>
       </c>
       <c r="B59">
-        <v>678394</v>
+        <v>686752</v>
       </c>
       <c r="C59" t="s">
         <v>285</v>
@@ -1883,32 +1868,32 @@
     </row>
     <row r="60" spans="1:3">
       <c r="A60" t="s">
-        <v>61</v>
+        <v>56</v>
       </c>
       <c r="B60">
-        <v>450203</v>
+        <v>640455</v>
       </c>
       <c r="C60" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="61" spans="1:3">
       <c r="A61" t="s">
-        <v>62</v>
+        <v>57</v>
       </c>
       <c r="B61">
-        <v>477132</v>
+        <v>663941</v>
       </c>
       <c r="C61" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
     </row>
     <row r="62" spans="1:3">
       <c r="A62" t="s">
-        <v>63</v>
+        <v>58</v>
       </c>
       <c r="B62">
-        <v>607067</v>
+        <v>805673</v>
       </c>
       <c r="C62" t="s">
         <v>285</v>
@@ -1916,10 +1901,10 @@
     </row>
     <row r="63" spans="1:3">
       <c r="A63" t="s">
-        <v>64</v>
+        <v>59</v>
       </c>
       <c r="B63">
-        <v>663436</v>
+        <v>681343</v>
       </c>
       <c r="C63" t="s">
         <v>285</v>
@@ -1927,10 +1912,10 @@
     </row>
     <row r="64" spans="1:3">
       <c r="A64" t="s">
-        <v>65</v>
+        <v>60</v>
       </c>
       <c r="B64">
-        <v>656876</v>
+        <v>690990</v>
       </c>
       <c r="C64" t="s">
         <v>285</v>
@@ -1938,10 +1923,10 @@
     </row>
     <row r="65" spans="1:3">
       <c r="A65" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="B65">
-        <v>656302</v>
+        <v>693645</v>
       </c>
       <c r="C65" t="s">
         <v>285</v>
@@ -1949,21 +1934,21 @@
     </row>
     <row r="66" spans="1:3">
       <c r="A66" t="s">
-        <v>67</v>
+        <v>62</v>
       </c>
       <c r="B66">
-        <v>664285</v>
+        <v>813349</v>
       </c>
       <c r="C66" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
     </row>
     <row r="67" spans="1:3">
       <c r="A67" t="s">
-        <v>68</v>
+        <v>63</v>
       </c>
       <c r="B67">
-        <v>668881</v>
+        <v>805123</v>
       </c>
       <c r="C67" t="s">
         <v>285</v>
@@ -1971,21 +1956,21 @@
     </row>
     <row r="68" spans="1:3">
       <c r="A68" t="s">
-        <v>69</v>
+        <v>64</v>
       </c>
       <c r="B68">
-        <v>622491</v>
+        <v>607074</v>
       </c>
       <c r="C68" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="69" spans="1:3">
       <c r="A69" t="s">
-        <v>70</v>
+        <v>65</v>
       </c>
       <c r="B69">
-        <v>622663</v>
+        <v>686218</v>
       </c>
       <c r="C69" t="s">
         <v>285</v>
@@ -1993,21 +1978,21 @@
     </row>
     <row r="70" spans="1:3">
       <c r="A70" t="s">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="B70">
-        <v>608331</v>
+        <v>592791</v>
       </c>
       <c r="C70" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
     </row>
     <row r="71" spans="1:3">
       <c r="A71" t="s">
-        <v>72</v>
+        <v>67</v>
       </c>
       <c r="B71">
-        <v>453286</v>
+        <v>671212</v>
       </c>
       <c r="C71" t="s">
         <v>285</v>
@@ -2015,10 +2000,10 @@
     </row>
     <row r="72" spans="1:3">
       <c r="A72" t="s">
-        <v>73</v>
+        <v>68</v>
       </c>
       <c r="B72">
-        <v>547179</v>
+        <v>680694</v>
       </c>
       <c r="C72" t="s">
         <v>285</v>
@@ -2026,32 +2011,32 @@
     </row>
     <row r="73" spans="1:3">
       <c r="A73" t="s">
-        <v>74</v>
+        <v>69</v>
       </c>
       <c r="B73">
-        <v>571578</v>
+        <v>669461</v>
       </c>
       <c r="C73" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
     </row>
     <row r="74" spans="1:3">
       <c r="A74" t="s">
-        <v>75</v>
+        <v>70</v>
       </c>
       <c r="B74">
-        <v>669194</v>
+        <v>680730</v>
       </c>
       <c r="C74" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="75" spans="1:3">
       <c r="A75" t="s">
-        <v>76</v>
+        <v>71</v>
       </c>
       <c r="B75">
-        <v>543243</v>
+        <v>680732</v>
       </c>
       <c r="C75" t="s">
         <v>285</v>
@@ -2059,10 +2044,10 @@
     </row>
     <row r="76" spans="1:3">
       <c r="A76" t="s">
-        <v>77</v>
+        <v>72</v>
       </c>
       <c r="B76">
-        <v>592836</v>
+        <v>675911</v>
       </c>
       <c r="C76" t="s">
         <v>285</v>
@@ -2070,10 +2055,10 @@
     </row>
     <row r="77" spans="1:3">
       <c r="A77" t="s">
-        <v>78</v>
+        <v>73</v>
       </c>
       <c r="B77">
-        <v>685299</v>
+        <v>668678</v>
       </c>
       <c r="C77" t="s">
         <v>285</v>
@@ -2081,10 +2066,10 @@
     </row>
     <row r="78" spans="1:3">
       <c r="A78" t="s">
-        <v>79</v>
+        <v>74</v>
       </c>
       <c r="B78">
-        <v>608372</v>
+        <v>641793</v>
       </c>
       <c r="C78" t="s">
         <v>285</v>
@@ -2092,10 +2077,10 @@
     </row>
     <row r="79" spans="1:3">
       <c r="A79" t="s">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="B79">
-        <v>694819</v>
+        <v>669920</v>
       </c>
       <c r="C79" t="s">
         <v>285</v>
@@ -2103,21 +2088,21 @@
     </row>
     <row r="80" spans="1:3">
       <c r="A80" t="s">
-        <v>81</v>
+        <v>76</v>
       </c>
       <c r="B80">
-        <v>800048</v>
+        <v>678906</v>
       </c>
       <c r="C80" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
     </row>
     <row r="81" spans="1:3">
       <c r="A81" t="s">
-        <v>82</v>
+        <v>77</v>
       </c>
       <c r="B81">
-        <v>696149</v>
+        <v>702056</v>
       </c>
       <c r="C81" t="s">
         <v>285</v>
@@ -2125,32 +2110,32 @@
     </row>
     <row r="82" spans="1:3">
       <c r="A82" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="B82">
-        <v>674841</v>
+        <v>800049</v>
       </c>
       <c r="C82" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
     </row>
     <row r="83" spans="1:3">
       <c r="A83" t="s">
-        <v>84</v>
+        <v>79</v>
       </c>
       <c r="B83">
-        <v>815083</v>
+        <v>641927</v>
       </c>
       <c r="C83" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
     </row>
     <row r="84" spans="1:3">
       <c r="A84" t="s">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="B84">
-        <v>687075</v>
+        <v>678394</v>
       </c>
       <c r="C84" t="s">
         <v>285</v>
@@ -2158,10 +2143,10 @@
     </row>
     <row r="85" spans="1:3">
       <c r="A85" t="s">
-        <v>86</v>
+        <v>81</v>
       </c>
       <c r="B85">
-        <v>669467</v>
+        <v>450203</v>
       </c>
       <c r="C85" t="s">
         <v>285</v>
@@ -2169,21 +2154,21 @@
     </row>
     <row r="86" spans="1:3">
       <c r="A86" t="s">
-        <v>87</v>
+        <v>82</v>
       </c>
       <c r="B86">
-        <v>663903</v>
+        <v>477132</v>
       </c>
       <c r="C86" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="87" spans="1:3">
       <c r="A87" t="s">
-        <v>88</v>
+        <v>83</v>
       </c>
       <c r="B87">
-        <v>694297</v>
+        <v>607067</v>
       </c>
       <c r="C87" t="s">
         <v>285</v>
@@ -2191,10 +2176,10 @@
     </row>
     <row r="88" spans="1:3">
       <c r="A88" t="s">
-        <v>89</v>
+        <v>84</v>
       </c>
       <c r="B88">
-        <v>605540</v>
+        <v>656876</v>
       </c>
       <c r="C88" t="s">
         <v>285</v>
@@ -2202,10 +2187,10 @@
     </row>
     <row r="89" spans="1:3">
       <c r="A89" t="s">
-        <v>90</v>
+        <v>85</v>
       </c>
       <c r="B89">
-        <v>682243</v>
+        <v>656302</v>
       </c>
       <c r="C89" t="s">
         <v>285</v>
@@ -2213,21 +2198,21 @@
     </row>
     <row r="90" spans="1:3">
       <c r="A90" t="s">
-        <v>91</v>
+        <v>86</v>
       </c>
       <c r="B90">
-        <v>605135</v>
+        <v>664285</v>
       </c>
       <c r="C90" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="91" spans="1:3">
       <c r="A91" t="s">
-        <v>92</v>
+        <v>87</v>
       </c>
       <c r="B91">
-        <v>686613</v>
+        <v>668881</v>
       </c>
       <c r="C91" t="s">
         <v>285</v>
@@ -2235,10 +2220,10 @@
     </row>
     <row r="92" spans="1:3">
       <c r="A92" t="s">
-        <v>93</v>
+        <v>88</v>
       </c>
       <c r="B92">
-        <v>694462</v>
+        <v>622663</v>
       </c>
       <c r="C92" t="s">
         <v>285</v>
@@ -2246,21 +2231,21 @@
     </row>
     <row r="93" spans="1:3">
       <c r="A93" t="s">
-        <v>94</v>
+        <v>89</v>
       </c>
       <c r="B93">
-        <v>669372</v>
+        <v>608331</v>
       </c>
       <c r="C93" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="94" spans="1:3">
       <c r="A94" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="B94">
-        <v>594798</v>
+        <v>453286</v>
       </c>
       <c r="C94" t="s">
         <v>285</v>
@@ -2268,32 +2253,32 @@
     </row>
     <row r="95" spans="1:3">
       <c r="A95" t="s">
-        <v>96</v>
+        <v>91</v>
       </c>
       <c r="B95">
-        <v>666200</v>
+        <v>547179</v>
       </c>
       <c r="C95" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
     </row>
     <row r="96" spans="1:3">
       <c r="A96" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
       <c r="B96">
-        <v>657746</v>
+        <v>571578</v>
       </c>
       <c r="C96" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="97" spans="1:3">
       <c r="A97" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
       <c r="B97">
-        <v>434378</v>
+        <v>669194</v>
       </c>
       <c r="C97" t="s">
         <v>285</v>
@@ -2301,10 +2286,10 @@
     </row>
     <row r="98" spans="1:3">
       <c r="A98" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
       <c r="B98">
-        <v>608337</v>
+        <v>543243</v>
       </c>
       <c r="C98" t="s">
         <v>285</v>
@@ -2312,21 +2297,21 @@
     </row>
     <row r="99" spans="1:3">
       <c r="A99" t="s">
-        <v>100</v>
+        <v>95</v>
       </c>
       <c r="B99">
-        <v>527048</v>
+        <v>685299</v>
       </c>
       <c r="C99" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
     </row>
     <row r="100" spans="1:3">
       <c r="A100" t="s">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="B100">
-        <v>656605</v>
+        <v>694819</v>
       </c>
       <c r="C100" t="s">
         <v>285</v>
@@ -2334,21 +2319,21 @@
     </row>
     <row r="101" spans="1:3">
       <c r="A101" t="s">
-        <v>102</v>
+        <v>97</v>
       </c>
       <c r="B101">
-        <v>681190</v>
+        <v>800048</v>
       </c>
       <c r="C101" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="102" spans="1:3">
       <c r="A102" t="s">
-        <v>103</v>
+        <v>98</v>
       </c>
       <c r="B102">
-        <v>645261</v>
+        <v>696149</v>
       </c>
       <c r="C102" t="s">
         <v>285</v>
@@ -2356,54 +2341,54 @@
     </row>
     <row r="103" spans="1:3">
       <c r="A103" t="s">
-        <v>104</v>
+        <v>99</v>
       </c>
       <c r="B103">
-        <v>669358</v>
+        <v>674841</v>
       </c>
       <c r="C103" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="104" spans="1:3">
       <c r="A104" t="s">
-        <v>105</v>
+        <v>100</v>
       </c>
       <c r="B104">
-        <v>676440</v>
+        <v>815083</v>
       </c>
       <c r="C104" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="105" spans="1:3">
       <c r="A105" t="s">
-        <v>106</v>
+        <v>101</v>
       </c>
       <c r="B105">
-        <v>669373</v>
+        <v>687075</v>
       </c>
       <c r="C105" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
     </row>
     <row r="106" spans="1:3">
       <c r="A106" t="s">
-        <v>107</v>
+        <v>102</v>
       </c>
       <c r="B106">
-        <v>669432</v>
+        <v>669467</v>
       </c>
       <c r="C106" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
     </row>
     <row r="107" spans="1:3">
       <c r="A107" t="s">
-        <v>108</v>
+        <v>103</v>
       </c>
       <c r="B107">
-        <v>808967</v>
+        <v>663903</v>
       </c>
       <c r="C107" t="s">
         <v>285</v>
@@ -2411,21 +2396,21 @@
     </row>
     <row r="108" spans="1:3">
       <c r="A108" t="s">
-        <v>109</v>
+        <v>104</v>
       </c>
       <c r="B108">
-        <v>579328</v>
+        <v>694297</v>
       </c>
       <c r="C108" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
     </row>
     <row r="109" spans="1:3">
       <c r="A109" t="s">
-        <v>110</v>
+        <v>105</v>
       </c>
       <c r="B109">
-        <v>695418</v>
+        <v>605540</v>
       </c>
       <c r="C109" t="s">
         <v>285</v>
@@ -2433,10 +2418,10 @@
     </row>
     <row r="110" spans="1:3">
       <c r="A110" t="s">
-        <v>111</v>
+        <v>106</v>
       </c>
       <c r="B110">
-        <v>663568</v>
+        <v>682243</v>
       </c>
       <c r="C110" t="s">
         <v>285</v>
@@ -2444,10 +2429,10 @@
     </row>
     <row r="111" spans="1:3">
       <c r="A111" t="s">
-        <v>112</v>
+        <v>107</v>
       </c>
       <c r="B111">
-        <v>685326</v>
+        <v>686613</v>
       </c>
       <c r="C111" t="s">
         <v>285</v>
@@ -2455,10 +2440,10 @@
     </row>
     <row r="112" spans="1:3">
       <c r="A112" t="s">
-        <v>113</v>
+        <v>108</v>
       </c>
       <c r="B112">
-        <v>804636</v>
+        <v>694462</v>
       </c>
       <c r="C112" t="s">
         <v>285</v>
@@ -2466,21 +2451,21 @@
     </row>
     <row r="113" spans="1:3">
       <c r="A113" t="s">
-        <v>114</v>
+        <v>109</v>
       </c>
       <c r="B113">
-        <v>656849</v>
+        <v>669372</v>
       </c>
       <c r="C113" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
     </row>
     <row r="114" spans="1:3">
       <c r="A114" t="s">
-        <v>115</v>
+        <v>110</v>
       </c>
       <c r="B114">
-        <v>668909</v>
+        <v>594798</v>
       </c>
       <c r="C114" t="s">
         <v>285</v>
@@ -2488,21 +2473,21 @@
     </row>
     <row r="115" spans="1:3">
       <c r="A115" t="s">
-        <v>116</v>
+        <v>111</v>
       </c>
       <c r="B115">
-        <v>656427</v>
+        <v>666200</v>
       </c>
       <c r="C115" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="116" spans="1:3">
       <c r="A116" t="s">
-        <v>117</v>
+        <v>112</v>
       </c>
       <c r="B116">
-        <v>665871</v>
+        <v>657746</v>
       </c>
       <c r="C116" t="s">
         <v>285</v>
@@ -2510,10 +2495,10 @@
     </row>
     <row r="117" spans="1:3">
       <c r="A117" t="s">
-        <v>118</v>
+        <v>113</v>
       </c>
       <c r="B117">
-        <v>670912</v>
+        <v>608337</v>
       </c>
       <c r="C117" t="s">
         <v>285</v>
@@ -2521,21 +2506,21 @@
     </row>
     <row r="118" spans="1:3">
       <c r="A118" t="s">
-        <v>119</v>
+        <v>114</v>
       </c>
       <c r="B118">
-        <v>667755</v>
+        <v>527048</v>
       </c>
       <c r="C118" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="119" spans="1:3">
       <c r="A119" t="s">
-        <v>120</v>
+        <v>115</v>
       </c>
       <c r="B119">
-        <v>601713</v>
+        <v>656605</v>
       </c>
       <c r="C119" t="s">
         <v>285</v>
@@ -2543,10 +2528,10 @@
     </row>
     <row r="120" spans="1:3">
       <c r="A120" t="s">
-        <v>121</v>
+        <v>116</v>
       </c>
       <c r="B120">
-        <v>641154</v>
+        <v>681190</v>
       </c>
       <c r="C120" t="s">
         <v>285</v>
@@ -2554,10 +2539,10 @@
     </row>
     <row r="121" spans="1:3">
       <c r="A121" t="s">
-        <v>122</v>
+        <v>117</v>
       </c>
       <c r="B121">
-        <v>682990</v>
+        <v>645261</v>
       </c>
       <c r="C121" t="s">
         <v>285</v>
@@ -2565,10 +2550,10 @@
     </row>
     <row r="122" spans="1:3">
       <c r="A122" t="s">
-        <v>123</v>
+        <v>118</v>
       </c>
       <c r="B122">
-        <v>678368</v>
+        <v>669358</v>
       </c>
       <c r="C122" t="s">
         <v>285</v>
@@ -2576,65 +2561,65 @@
     </row>
     <row r="123" spans="1:3">
       <c r="A123" t="s">
-        <v>124</v>
+        <v>119</v>
       </c>
       <c r="B123">
-        <v>676467</v>
+        <v>676440</v>
       </c>
       <c r="C123" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
     </row>
     <row r="124" spans="1:3">
       <c r="A124" t="s">
-        <v>125</v>
+        <v>120</v>
       </c>
       <c r="B124">
-        <v>693313</v>
+        <v>669373</v>
       </c>
       <c r="C124" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="125" spans="1:3">
       <c r="A125" t="s">
-        <v>126</v>
+        <v>121</v>
       </c>
       <c r="B125">
-        <v>693855</v>
+        <v>669432</v>
       </c>
       <c r="C125" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
     </row>
     <row r="126" spans="1:3">
       <c r="A126" t="s">
-        <v>127</v>
+        <v>122</v>
       </c>
       <c r="B126">
-        <v>801139</v>
+        <v>808967</v>
       </c>
       <c r="C126" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
     </row>
     <row r="127" spans="1:3">
       <c r="A127" t="s">
-        <v>128</v>
+        <v>123</v>
       </c>
       <c r="B127">
-        <v>686930</v>
+        <v>579328</v>
       </c>
       <c r="C127" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="128" spans="1:3">
       <c r="A128" t="s">
-        <v>129</v>
+        <v>124</v>
       </c>
       <c r="B128">
-        <v>607192</v>
+        <v>695418</v>
       </c>
       <c r="C128" t="s">
         <v>285</v>
@@ -2642,21 +2627,21 @@
     </row>
     <row r="129" spans="1:3">
       <c r="A129" t="s">
-        <v>130</v>
+        <v>125</v>
       </c>
       <c r="B129">
-        <v>605483</v>
+        <v>663568</v>
       </c>
       <c r="C129" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
     </row>
     <row r="130" spans="1:3">
       <c r="A130" t="s">
-        <v>131</v>
+        <v>126</v>
       </c>
       <c r="B130">
-        <v>664299</v>
+        <v>685326</v>
       </c>
       <c r="C130" t="s">
         <v>285</v>
@@ -2664,10 +2649,10 @@
     </row>
     <row r="131" spans="1:3">
       <c r="A131" t="s">
-        <v>132</v>
+        <v>127</v>
       </c>
       <c r="B131">
-        <v>686563</v>
+        <v>804636</v>
       </c>
       <c r="C131" t="s">
         <v>285</v>
@@ -2675,32 +2660,32 @@
     </row>
     <row r="132" spans="1:3">
       <c r="A132" t="s">
-        <v>133</v>
+        <v>128</v>
       </c>
       <c r="B132">
-        <v>543294</v>
+        <v>656849</v>
       </c>
       <c r="C132" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="133" spans="1:3">
       <c r="A133" t="s">
-        <v>134</v>
+        <v>129</v>
       </c>
       <c r="B133">
-        <v>671106</v>
+        <v>668909</v>
       </c>
       <c r="C133" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
     </row>
     <row r="134" spans="1:3">
       <c r="A134" t="s">
-        <v>135</v>
+        <v>130</v>
       </c>
       <c r="B134">
-        <v>671737</v>
+        <v>656427</v>
       </c>
       <c r="C134" t="s">
         <v>285</v>
@@ -2708,21 +2693,21 @@
     </row>
     <row r="135" spans="1:3">
       <c r="A135" t="s">
-        <v>136</v>
+        <v>131</v>
       </c>
       <c r="B135">
-        <v>702070</v>
+        <v>665871</v>
       </c>
       <c r="C135" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
     </row>
     <row r="136" spans="1:3">
       <c r="A136" t="s">
-        <v>137</v>
+        <v>132</v>
       </c>
       <c r="B136">
-        <v>605400</v>
+        <v>670912</v>
       </c>
       <c r="C136" t="s">
         <v>285</v>
@@ -2730,10 +2715,10 @@
     </row>
     <row r="137" spans="1:3">
       <c r="A137" t="s">
-        <v>138</v>
+        <v>133</v>
       </c>
       <c r="B137">
-        <v>605288</v>
+        <v>667755</v>
       </c>
       <c r="C137" t="s">
         <v>285</v>
@@ -2741,10 +2726,10 @@
     </row>
     <row r="138" spans="1:3">
       <c r="A138" t="s">
-        <v>139</v>
+        <v>134</v>
       </c>
       <c r="B138">
-        <v>693821</v>
+        <v>601713</v>
       </c>
       <c r="C138" t="s">
         <v>285</v>
@@ -2752,21 +2737,21 @@
     </row>
     <row r="139" spans="1:3">
       <c r="A139" t="s">
-        <v>140</v>
+        <v>135</v>
       </c>
       <c r="B139">
-        <v>700249</v>
+        <v>641154</v>
       </c>
       <c r="C139" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
     </row>
     <row r="140" spans="1:3">
       <c r="A140" t="s">
-        <v>141</v>
+        <v>136</v>
       </c>
       <c r="B140">
-        <v>605280</v>
+        <v>682990</v>
       </c>
       <c r="C140" t="s">
         <v>285</v>
@@ -2774,10 +2759,10 @@
     </row>
     <row r="141" spans="1:3">
       <c r="A141" t="s">
-        <v>142</v>
+        <v>137</v>
       </c>
       <c r="B141">
-        <v>669160</v>
+        <v>678368</v>
       </c>
       <c r="C141" t="s">
         <v>285</v>
@@ -2785,54 +2770,54 @@
     </row>
     <row r="142" spans="1:3">
       <c r="A142" t="s">
-        <v>143</v>
+        <v>138</v>
       </c>
       <c r="B142">
-        <v>608566</v>
+        <v>676467</v>
       </c>
       <c r="C142" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="143" spans="1:3">
       <c r="A143" t="s">
-        <v>144</v>
+        <v>139</v>
       </c>
       <c r="B143">
-        <v>500779</v>
+        <v>693313</v>
       </c>
       <c r="C143" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
     </row>
     <row r="144" spans="1:3">
       <c r="A144" t="s">
-        <v>145</v>
+        <v>140</v>
       </c>
       <c r="B144">
-        <v>641482</v>
+        <v>693855</v>
       </c>
       <c r="C144" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
     </row>
     <row r="145" spans="1:3">
       <c r="A145" t="s">
-        <v>146</v>
+        <v>141</v>
       </c>
       <c r="B145">
-        <v>592662</v>
+        <v>801139</v>
       </c>
       <c r="C145" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
     </row>
     <row r="146" spans="1:3">
       <c r="A146" t="s">
-        <v>147</v>
+        <v>142</v>
       </c>
       <c r="B146">
-        <v>669456</v>
+        <v>686930</v>
       </c>
       <c r="C146" t="s">
         <v>285</v>
@@ -2840,10 +2825,10 @@
     </row>
     <row r="147" spans="1:3">
       <c r="A147" t="s">
-        <v>148</v>
+        <v>143</v>
       </c>
       <c r="B147">
-        <v>701542</v>
+        <v>607192</v>
       </c>
       <c r="C147" t="s">
         <v>285</v>
@@ -2851,21 +2836,21 @@
     </row>
     <row r="148" spans="1:3">
       <c r="A148" t="s">
-        <v>149</v>
+        <v>144</v>
       </c>
       <c r="B148">
-        <v>686701</v>
+        <v>605483</v>
       </c>
       <c r="C148" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="149" spans="1:3">
       <c r="A149" t="s">
-        <v>150</v>
+        <v>145</v>
       </c>
       <c r="B149">
-        <v>672782</v>
+        <v>664299</v>
       </c>
       <c r="C149" t="s">
         <v>285</v>
@@ -2873,10 +2858,10 @@
     </row>
     <row r="150" spans="1:3">
       <c r="A150" t="s">
-        <v>151</v>
+        <v>146</v>
       </c>
       <c r="B150">
-        <v>693433</v>
+        <v>686563</v>
       </c>
       <c r="C150" t="s">
         <v>285</v>
@@ -2884,10 +2869,10 @@
     </row>
     <row r="151" spans="1:3">
       <c r="A151" t="s">
-        <v>152</v>
+        <v>147</v>
       </c>
       <c r="B151">
-        <v>676917</v>
+        <v>543294</v>
       </c>
       <c r="C151" t="s">
         <v>285</v>
@@ -2895,43 +2880,43 @@
     </row>
     <row r="152" spans="1:3">
       <c r="A152" t="s">
-        <v>153</v>
+        <v>148</v>
       </c>
       <c r="B152">
-        <v>676979</v>
+        <v>671106</v>
       </c>
       <c r="C152" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
     </row>
     <row r="153" spans="1:3">
       <c r="A153" t="s">
-        <v>154</v>
+        <v>149</v>
       </c>
       <c r="B153">
-        <v>666214</v>
+        <v>671737</v>
       </c>
       <c r="C153" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
     </row>
     <row r="154" spans="1:3">
       <c r="A154" t="s">
-        <v>155</v>
+        <v>150</v>
       </c>
       <c r="B154">
-        <v>657277</v>
+        <v>702070</v>
       </c>
       <c r="C154" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="155" spans="1:3">
       <c r="A155" t="s">
-        <v>156</v>
+        <v>151</v>
       </c>
       <c r="B155">
-        <v>571945</v>
+        <v>605400</v>
       </c>
       <c r="C155" t="s">
         <v>285</v>
@@ -2939,10 +2924,10 @@
     </row>
     <row r="156" spans="1:3">
       <c r="A156" t="s">
-        <v>157</v>
+        <v>152</v>
       </c>
       <c r="B156">
-        <v>622503</v>
+        <v>605288</v>
       </c>
       <c r="C156" t="s">
         <v>285</v>
@@ -2950,32 +2935,32 @@
     </row>
     <row r="157" spans="1:3">
       <c r="A157" t="s">
-        <v>158</v>
+        <v>153</v>
       </c>
       <c r="B157">
-        <v>666157</v>
+        <v>700249</v>
       </c>
       <c r="C157" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
     </row>
     <row r="158" spans="1:3">
       <c r="A158" t="s">
-        <v>159</v>
+        <v>154</v>
       </c>
       <c r="B158">
-        <v>684007</v>
+        <v>669160</v>
       </c>
       <c r="C158" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
     </row>
     <row r="159" spans="1:3">
       <c r="A159" t="s">
-        <v>160</v>
+        <v>155</v>
       </c>
       <c r="B159">
-        <v>677944</v>
+        <v>608566</v>
       </c>
       <c r="C159" t="s">
         <v>285</v>
@@ -2983,54 +2968,54 @@
     </row>
     <row r="160" spans="1:3">
       <c r="A160" t="s">
-        <v>161</v>
+        <v>156</v>
       </c>
       <c r="B160">
-        <v>669330</v>
+        <v>500779</v>
       </c>
       <c r="C160" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="161" spans="1:3">
       <c r="A161" t="s">
-        <v>162</v>
+        <v>157</v>
       </c>
       <c r="B161">
-        <v>506433</v>
+        <v>641482</v>
       </c>
       <c r="C161" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="162" spans="1:3">
       <c r="A162" t="s">
-        <v>163</v>
+        <v>158</v>
       </c>
       <c r="B162">
-        <v>687830</v>
+        <v>592662</v>
       </c>
       <c r="C162" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="163" spans="1:3">
       <c r="A163" t="s">
-        <v>164</v>
+        <v>159</v>
       </c>
       <c r="B163">
-        <v>656641</v>
+        <v>669456</v>
       </c>
       <c r="C163" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
     </row>
     <row r="164" spans="1:3">
       <c r="A164" t="s">
-        <v>165</v>
+        <v>160</v>
       </c>
       <c r="B164">
-        <v>690997</v>
+        <v>701542</v>
       </c>
       <c r="C164" t="s">
         <v>285</v>
@@ -3038,26 +3023,32 @@
     </row>
     <row r="165" spans="1:3">
       <c r="A165" t="s">
-        <v>166</v>
+        <v>161</v>
       </c>
       <c r="B165">
-        <v>669060</v>
+        <v>686701</v>
       </c>
       <c r="C165" t="s">
         <v>285</v>
       </c>
     </row>
     <row r="166" spans="1:3">
+      <c r="A166" t="s">
+        <v>162</v>
+      </c>
+      <c r="B166">
+        <v>672782</v>
+      </c>
       <c r="C166" t="s">
         <v>285</v>
       </c>
     </row>
     <row r="167" spans="1:3">
       <c r="A167" t="s">
-        <v>167</v>
+        <v>163</v>
       </c>
       <c r="B167">
-        <v>801403</v>
+        <v>693433</v>
       </c>
       <c r="C167" t="s">
         <v>285</v>
@@ -3065,10 +3056,10 @@
     </row>
     <row r="168" spans="1:3">
       <c r="A168" t="s">
-        <v>168</v>
+        <v>164</v>
       </c>
       <c r="B168">
-        <v>806960</v>
+        <v>676917</v>
       </c>
       <c r="C168" t="s">
         <v>285</v>
@@ -3076,43 +3067,43 @@
     </row>
     <row r="169" spans="1:3">
       <c r="A169" t="s">
-        <v>169</v>
+        <v>165</v>
       </c>
       <c r="B169">
-        <v>678215</v>
+        <v>676979</v>
       </c>
       <c r="C169" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="170" spans="1:3">
       <c r="A170" t="s">
-        <v>170</v>
+        <v>166</v>
       </c>
       <c r="B170">
-        <v>673540</v>
+        <v>666214</v>
       </c>
       <c r="C170" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="171" spans="1:3">
       <c r="A171" t="s">
-        <v>171</v>
+        <v>167</v>
       </c>
       <c r="B171">
-        <v>606996</v>
+        <v>657277</v>
       </c>
       <c r="C171" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
     </row>
     <row r="172" spans="1:3">
       <c r="A172" t="s">
-        <v>172</v>
+        <v>168</v>
       </c>
       <c r="B172">
-        <v>665795</v>
+        <v>571945</v>
       </c>
       <c r="C172" t="s">
         <v>285</v>
@@ -3120,10 +3111,10 @@
     </row>
     <row r="173" spans="1:3">
       <c r="A173" t="s">
-        <v>173</v>
+        <v>169</v>
       </c>
       <c r="B173">
-        <v>681293</v>
+        <v>622503</v>
       </c>
       <c r="C173" t="s">
         <v>285</v>
@@ -3131,43 +3122,43 @@
     </row>
     <row r="174" spans="1:3">
       <c r="A174" t="s">
-        <v>174</v>
+        <v>170</v>
       </c>
       <c r="B174">
-        <v>663978</v>
+        <v>666157</v>
       </c>
       <c r="C174" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="175" spans="1:3">
       <c r="A175" t="s">
-        <v>175</v>
+        <v>171</v>
       </c>
       <c r="B175">
-        <v>607625</v>
+        <v>684007</v>
       </c>
       <c r="C175" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="176" spans="1:3">
       <c r="A176" t="s">
-        <v>176</v>
+        <v>172</v>
       </c>
       <c r="B176">
-        <v>542881</v>
+        <v>677944</v>
       </c>
       <c r="C176" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
     </row>
     <row r="177" spans="1:3">
       <c r="A177" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="B177">
-        <v>615698</v>
+        <v>669330</v>
       </c>
       <c r="C177" t="s">
         <v>285</v>
@@ -3175,10 +3166,10 @@
     </row>
     <row r="178" spans="1:3">
       <c r="A178" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="B178">
-        <v>650644</v>
+        <v>506433</v>
       </c>
       <c r="C178" t="s">
         <v>285</v>
@@ -3186,32 +3177,32 @@
     </row>
     <row r="179" spans="1:3">
       <c r="A179" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="B179">
-        <v>687931</v>
+        <v>687830</v>
       </c>
       <c r="C179" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
     </row>
     <row r="180" spans="1:3">
       <c r="A180" t="s">
-        <v>180</v>
+        <v>176</v>
       </c>
       <c r="B180">
-        <v>641778</v>
+        <v>656641</v>
       </c>
       <c r="C180" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
     </row>
     <row r="181" spans="1:3">
       <c r="A181" t="s">
-        <v>181</v>
+        <v>177</v>
       </c>
       <c r="B181">
-        <v>686799</v>
+        <v>690997</v>
       </c>
       <c r="C181" t="s">
         <v>285</v>
@@ -3219,10 +3210,10 @@
     </row>
     <row r="182" spans="1:3">
       <c r="A182" t="s">
-        <v>182</v>
+        <v>178</v>
       </c>
       <c r="B182">
-        <v>672710</v>
+        <v>669060</v>
       </c>
       <c r="C182" t="s">
         <v>285</v>
@@ -3230,10 +3221,10 @@
     </row>
     <row r="183" spans="1:3">
       <c r="A183" t="s">
-        <v>183</v>
+        <v>179</v>
       </c>
       <c r="B183">
-        <v>687473</v>
+        <v>801403</v>
       </c>
       <c r="C183" t="s">
         <v>285</v>
@@ -3241,10 +3232,10 @@
     </row>
     <row r="184" spans="1:3">
       <c r="A184" t="s">
-        <v>184</v>
+        <v>180</v>
       </c>
       <c r="B184">
-        <v>607259</v>
+        <v>806960</v>
       </c>
       <c r="C184" t="s">
         <v>285</v>
@@ -3252,10 +3243,10 @@
     </row>
     <row r="185" spans="1:3">
       <c r="A185" t="s">
-        <v>185</v>
+        <v>181</v>
       </c>
       <c r="B185">
-        <v>674370</v>
+        <v>678215</v>
       </c>
       <c r="C185" t="s">
         <v>285</v>
@@ -3263,65 +3254,65 @@
     </row>
     <row r="186" spans="1:3">
       <c r="A186" t="s">
-        <v>186</v>
+        <v>182</v>
       </c>
       <c r="B186">
-        <v>676664</v>
+        <v>673540</v>
       </c>
       <c r="C186" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
     </row>
     <row r="187" spans="1:3">
       <c r="A187" t="s">
-        <v>187</v>
+        <v>183</v>
       </c>
       <c r="B187">
-        <v>690916</v>
+        <v>606996</v>
       </c>
       <c r="C187" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="188" spans="1:3">
       <c r="A188" t="s">
-        <v>188</v>
+        <v>184</v>
       </c>
       <c r="B188">
-        <v>688107</v>
+        <v>681293</v>
       </c>
       <c r="C188" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
     </row>
     <row r="189" spans="1:3">
       <c r="A189" t="s">
-        <v>189</v>
+        <v>185</v>
       </c>
       <c r="B189">
-        <v>682052</v>
+        <v>607625</v>
       </c>
       <c r="C189" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
     </row>
     <row r="190" spans="1:3">
       <c r="A190" t="s">
-        <v>190</v>
+        <v>186</v>
       </c>
       <c r="B190">
-        <v>676083</v>
+        <v>542881</v>
       </c>
       <c r="C190" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="191" spans="1:3">
       <c r="A191" t="s">
-        <v>191</v>
+        <v>187</v>
       </c>
       <c r="B191">
-        <v>690953</v>
+        <v>615698</v>
       </c>
       <c r="C191" t="s">
         <v>285</v>
@@ -3329,10 +3320,10 @@
     </row>
     <row r="192" spans="1:3">
       <c r="A192" t="s">
-        <v>192</v>
+        <v>188</v>
       </c>
       <c r="B192">
-        <v>681347</v>
+        <v>650644</v>
       </c>
       <c r="C192" t="s">
         <v>285</v>
@@ -3340,32 +3331,32 @@
     </row>
     <row r="193" spans="1:3">
       <c r="A193" t="s">
-        <v>193</v>
+        <v>189</v>
       </c>
       <c r="B193">
-        <v>682929</v>
+        <v>687931</v>
       </c>
       <c r="C193" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="194" spans="1:3">
       <c r="A194" t="s">
-        <v>194</v>
+        <v>190</v>
       </c>
       <c r="B194">
-        <v>570632</v>
+        <v>641778</v>
       </c>
       <c r="C194" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="195" spans="1:3">
       <c r="A195" t="s">
-        <v>195</v>
+        <v>191</v>
       </c>
       <c r="B195">
-        <v>687064</v>
+        <v>686799</v>
       </c>
       <c r="C195" t="s">
         <v>285</v>
@@ -3373,10 +3364,10 @@
     </row>
     <row r="196" spans="1:3">
       <c r="A196" t="s">
-        <v>196</v>
+        <v>192</v>
       </c>
       <c r="B196">
-        <v>678022</v>
+        <v>672710</v>
       </c>
       <c r="C196" t="s">
         <v>285</v>
@@ -3384,10 +3375,10 @@
     </row>
     <row r="197" spans="1:3">
       <c r="A197" t="s">
-        <v>197</v>
+        <v>193</v>
       </c>
       <c r="B197">
-        <v>689017</v>
+        <v>687473</v>
       </c>
       <c r="C197" t="s">
         <v>285</v>
@@ -3395,29 +3386,32 @@
     </row>
     <row r="198" spans="1:3">
       <c r="A198" t="s">
-        <v>198</v>
+        <v>194</v>
       </c>
       <c r="B198">
-        <v>596295</v>
+        <v>674370</v>
       </c>
       <c r="C198" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
     </row>
     <row r="199" spans="1:3">
       <c r="A199" t="s">
-        <v>41</v>
+        <v>195</v>
+      </c>
+      <c r="B199">
+        <v>676664</v>
       </c>
       <c r="C199" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="200" spans="1:3">
       <c r="A200" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="B200">
-        <v>621111</v>
+        <v>690916</v>
       </c>
       <c r="C200" t="s">
         <v>285</v>
@@ -3425,32 +3419,32 @@
     </row>
     <row r="201" spans="1:3">
       <c r="A201" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="B201">
-        <v>694477</v>
+        <v>688107</v>
       </c>
       <c r="C201" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="202" spans="1:3">
       <c r="A202" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="B202">
-        <v>571760</v>
+        <v>676083</v>
       </c>
       <c r="C202" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
     </row>
     <row r="203" spans="1:3">
       <c r="A203" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="B203">
-        <v>607200</v>
+        <v>690953</v>
       </c>
       <c r="C203" t="s">
         <v>285</v>
@@ -3458,10 +3452,10 @@
     </row>
     <row r="204" spans="1:3">
       <c r="A204" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="B204">
-        <v>543135</v>
+        <v>681347</v>
       </c>
       <c r="C204" t="s">
         <v>285</v>
@@ -3469,10 +3463,10 @@
     </row>
     <row r="205" spans="1:3">
       <c r="A205" t="s">
-        <v>204</v>
+        <v>201</v>
       </c>
       <c r="B205">
-        <v>471911</v>
+        <v>682929</v>
       </c>
       <c r="C205" t="s">
         <v>285</v>
@@ -3480,21 +3474,21 @@
     </row>
     <row r="206" spans="1:3">
       <c r="A206" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="B206">
-        <v>663559</v>
+        <v>570632</v>
       </c>
       <c r="C206" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
     </row>
     <row r="207" spans="1:3">
       <c r="A207" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="B207">
-        <v>647336</v>
+        <v>687064</v>
       </c>
       <c r="C207" t="s">
         <v>285</v>
@@ -3502,10 +3496,10 @@
     </row>
     <row r="208" spans="1:3">
       <c r="A208" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="B208">
-        <v>701519</v>
+        <v>678022</v>
       </c>
       <c r="C208" t="s">
         <v>285</v>
@@ -3513,21 +3507,18 @@
     </row>
     <row r="209" spans="1:3">
       <c r="A209" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="B209">
-        <v>677958</v>
+        <v>596295</v>
       </c>
       <c r="C209" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="210" spans="1:3">
       <c r="A210" t="s">
-        <v>209</v>
-      </c>
-      <c r="B210">
-        <v>573186</v>
+        <v>65</v>
       </c>
       <c r="C210" t="s">
         <v>285</v>
@@ -3535,32 +3526,32 @@
     </row>
     <row r="211" spans="1:3">
       <c r="A211" t="s">
-        <v>210</v>
+        <v>206</v>
       </c>
       <c r="B211">
-        <v>687922</v>
+        <v>694477</v>
       </c>
       <c r="C211" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
     </row>
     <row r="212" spans="1:3">
       <c r="A212" t="s">
-        <v>211</v>
+        <v>207</v>
       </c>
       <c r="B212">
-        <v>688138</v>
+        <v>571760</v>
       </c>
       <c r="C212" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="213" spans="1:3">
       <c r="A213" t="s">
-        <v>212</v>
+        <v>208</v>
       </c>
       <c r="B213">
-        <v>701487</v>
+        <v>607200</v>
       </c>
       <c r="C213" t="s">
         <v>285</v>
@@ -3568,10 +3559,10 @@
     </row>
     <row r="214" spans="1:3">
       <c r="A214" t="s">
-        <v>213</v>
+        <v>209</v>
       </c>
       <c r="B214">
-        <v>687134</v>
+        <v>543135</v>
       </c>
       <c r="C214" t="s">
         <v>285</v>
@@ -3579,10 +3570,10 @@
     </row>
     <row r="215" spans="1:3">
       <c r="A215" t="s">
-        <v>214</v>
+        <v>210</v>
       </c>
       <c r="B215">
-        <v>593423</v>
+        <v>471911</v>
       </c>
       <c r="C215" t="s">
         <v>285</v>
@@ -3590,21 +3581,21 @@
     </row>
     <row r="216" spans="1:3">
       <c r="A216" t="s">
-        <v>215</v>
+        <v>211</v>
       </c>
       <c r="B216">
-        <v>448179</v>
+        <v>663559</v>
       </c>
       <c r="C216" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
     </row>
     <row r="217" spans="1:3">
       <c r="A217" t="s">
-        <v>216</v>
+        <v>212</v>
       </c>
       <c r="B217">
-        <v>621107</v>
+        <v>701519</v>
       </c>
       <c r="C217" t="s">
         <v>285</v>
@@ -3612,10 +3603,10 @@
     </row>
     <row r="218" spans="1:3">
       <c r="A218" t="s">
-        <v>217</v>
+        <v>213</v>
       </c>
       <c r="B218">
-        <v>695505</v>
+        <v>677958</v>
       </c>
       <c r="C218" t="s">
         <v>285</v>
@@ -3623,10 +3614,10 @@
     </row>
     <row r="219" spans="1:3">
       <c r="A219" t="s">
-        <v>218</v>
+        <v>214</v>
       </c>
       <c r="B219">
-        <v>675512</v>
+        <v>573186</v>
       </c>
       <c r="C219" t="s">
         <v>285</v>
@@ -3634,21 +3625,21 @@
     </row>
     <row r="220" spans="1:3">
       <c r="A220" t="s">
-        <v>219</v>
+        <v>215</v>
       </c>
       <c r="B220">
-        <v>676962</v>
+        <v>687922</v>
       </c>
       <c r="C220" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="221" spans="1:3">
       <c r="A221" t="s">
-        <v>220</v>
+        <v>216</v>
       </c>
       <c r="B221">
-        <v>554430</v>
+        <v>688138</v>
       </c>
       <c r="C221" t="s">
         <v>285</v>
@@ -3656,10 +3647,10 @@
     </row>
     <row r="222" spans="1:3">
       <c r="A222" t="s">
-        <v>221</v>
+        <v>217</v>
       </c>
       <c r="B222">
-        <v>656550</v>
+        <v>701487</v>
       </c>
       <c r="C222" t="s">
         <v>285</v>
@@ -3667,21 +3658,21 @@
     </row>
     <row r="223" spans="1:3">
       <c r="A223" t="s">
-        <v>222</v>
+        <v>218</v>
       </c>
       <c r="B223">
-        <v>663460</v>
+        <v>687134</v>
       </c>
       <c r="C223" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
     </row>
     <row r="224" spans="1:3">
       <c r="A224" t="s">
-        <v>223</v>
+        <v>219</v>
       </c>
       <c r="B224">
-        <v>669721</v>
+        <v>593423</v>
       </c>
       <c r="C224" t="s">
         <v>285</v>
@@ -3689,21 +3680,21 @@
     </row>
     <row r="225" spans="1:3">
       <c r="A225" t="s">
-        <v>224</v>
+        <v>220</v>
       </c>
       <c r="B225">
-        <v>701581</v>
+        <v>448179</v>
       </c>
       <c r="C225" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="226" spans="1:3">
       <c r="A226" t="s">
-        <v>225</v>
+        <v>221</v>
       </c>
       <c r="B226">
-        <v>806185</v>
+        <v>621107</v>
       </c>
       <c r="C226" t="s">
         <v>285</v>
@@ -3711,21 +3702,21 @@
     </row>
     <row r="227" spans="1:3">
       <c r="A227" t="s">
-        <v>226</v>
+        <v>222</v>
       </c>
       <c r="B227">
-        <v>687888</v>
+        <v>675512</v>
       </c>
       <c r="C227" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
     </row>
     <row r="228" spans="1:3">
       <c r="A228" t="s">
-        <v>227</v>
+        <v>223</v>
       </c>
       <c r="B228">
-        <v>681857</v>
+        <v>676962</v>
       </c>
       <c r="C228" t="s">
         <v>285</v>
@@ -3733,10 +3724,10 @@
     </row>
     <row r="229" spans="1:3">
       <c r="A229" t="s">
-        <v>228</v>
+        <v>224</v>
       </c>
       <c r="B229">
-        <v>666171</v>
+        <v>554430</v>
       </c>
       <c r="C229" t="s">
         <v>285</v>
@@ -3744,10 +3735,10 @@
     </row>
     <row r="230" spans="1:3">
       <c r="A230" t="s">
-        <v>229</v>
+        <v>225</v>
       </c>
       <c r="B230">
-        <v>663795</v>
+        <v>656550</v>
       </c>
       <c r="C230" t="s">
         <v>285</v>
@@ -3755,32 +3746,32 @@
     </row>
     <row r="231" spans="1:3">
       <c r="A231" t="s">
-        <v>230</v>
+        <v>226</v>
       </c>
       <c r="B231">
-        <v>696136</v>
+        <v>669721</v>
       </c>
       <c r="C231" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
     </row>
     <row r="232" spans="1:3">
       <c r="A232" t="s">
-        <v>231</v>
+        <v>227</v>
       </c>
       <c r="B232">
-        <v>680736</v>
+        <v>701581</v>
       </c>
       <c r="C232" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
     </row>
     <row r="233" spans="1:3">
       <c r="A233" t="s">
-        <v>232</v>
+        <v>228</v>
       </c>
       <c r="B233">
-        <v>642216</v>
+        <v>806185</v>
       </c>
       <c r="C233" t="s">
         <v>285</v>
@@ -3788,21 +3779,21 @@
     </row>
     <row r="234" spans="1:3">
       <c r="A234" t="s">
-        <v>233</v>
+        <v>229</v>
       </c>
       <c r="B234">
-        <v>621112</v>
+        <v>687888</v>
       </c>
       <c r="C234" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="235" spans="1:3">
       <c r="A235" t="s">
-        <v>234</v>
+        <v>230</v>
       </c>
       <c r="B235">
-        <v>680885</v>
+        <v>681857</v>
       </c>
       <c r="C235" t="s">
         <v>285</v>
@@ -3810,10 +3801,10 @@
     </row>
     <row r="236" spans="1:3">
       <c r="A236" t="s">
-        <v>235</v>
+        <v>231</v>
       </c>
       <c r="B236">
-        <v>605513</v>
+        <v>666171</v>
       </c>
       <c r="C236" t="s">
         <v>285</v>
@@ -3821,43 +3812,43 @@
     </row>
     <row r="237" spans="1:3">
       <c r="A237" t="s">
-        <v>236</v>
+        <v>232</v>
       </c>
       <c r="B237">
-        <v>641302</v>
+        <v>663795</v>
       </c>
       <c r="C237" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
     </row>
     <row r="238" spans="1:3">
       <c r="A238" t="s">
-        <v>237</v>
+        <v>233</v>
       </c>
       <c r="B238">
-        <v>690928</v>
+        <v>696136</v>
       </c>
       <c r="C238" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="239" spans="1:3">
       <c r="A239" t="s">
-        <v>238</v>
+        <v>234</v>
       </c>
       <c r="B239">
-        <v>694918</v>
+        <v>680736</v>
       </c>
       <c r="C239" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="240" spans="1:3">
       <c r="A240" t="s">
-        <v>239</v>
+        <v>235</v>
       </c>
       <c r="B240">
-        <v>800311</v>
+        <v>642216</v>
       </c>
       <c r="C240" t="s">
         <v>285</v>
@@ -3865,10 +3856,10 @@
     </row>
     <row r="241" spans="1:3">
       <c r="A241" t="s">
-        <v>240</v>
+        <v>236</v>
       </c>
       <c r="B241">
-        <v>592866</v>
+        <v>621112</v>
       </c>
       <c r="C241" t="s">
         <v>285</v>
@@ -3876,10 +3867,10 @@
     </row>
     <row r="242" spans="1:3">
       <c r="A242" t="s">
-        <v>241</v>
+        <v>237</v>
       </c>
       <c r="B242">
-        <v>678024</v>
+        <v>680885</v>
       </c>
       <c r="C242" t="s">
         <v>285</v>
@@ -3887,32 +3878,32 @@
     </row>
     <row r="243" spans="1:3">
       <c r="A243" t="s">
-        <v>242</v>
+        <v>238</v>
       </c>
       <c r="B243">
-        <v>642232</v>
+        <v>605513</v>
       </c>
       <c r="C243" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
     </row>
     <row r="244" spans="1:3">
       <c r="A244" t="s">
-        <v>243</v>
+        <v>239</v>
       </c>
       <c r="B244">
-        <v>669422</v>
+        <v>641302</v>
       </c>
       <c r="C244" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="245" spans="1:3">
       <c r="A245" t="s">
-        <v>244</v>
+        <v>240</v>
       </c>
       <c r="B245">
-        <v>657376</v>
+        <v>690928</v>
       </c>
       <c r="C245" t="s">
         <v>285</v>
@@ -3920,10 +3911,10 @@
     </row>
     <row r="246" spans="1:3">
       <c r="A246" t="s">
-        <v>245</v>
+        <v>241</v>
       </c>
       <c r="B246">
-        <v>676508</v>
+        <v>694918</v>
       </c>
       <c r="C246" t="s">
         <v>285</v>
@@ -3931,21 +3922,21 @@
     </row>
     <row r="247" spans="1:3">
       <c r="A247" t="s">
-        <v>246</v>
+        <v>242</v>
       </c>
       <c r="B247">
-        <v>687223</v>
+        <v>800311</v>
       </c>
       <c r="C247" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
     </row>
     <row r="248" spans="1:3">
       <c r="A248" t="s">
-        <v>247</v>
+        <v>243</v>
       </c>
       <c r="B248">
-        <v>656288</v>
+        <v>592866</v>
       </c>
       <c r="C248" t="s">
         <v>285</v>
@@ -3953,32 +3944,32 @@
     </row>
     <row r="249" spans="1:3">
       <c r="A249" t="s">
-        <v>248</v>
+        <v>244</v>
       </c>
       <c r="B249">
-        <v>690986</v>
+        <v>678024</v>
       </c>
       <c r="C249" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
     </row>
     <row r="250" spans="1:3">
       <c r="A250" t="s">
-        <v>249</v>
+        <v>245</v>
       </c>
       <c r="B250">
-        <v>687765</v>
+        <v>642232</v>
       </c>
       <c r="C250" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="251" spans="1:3">
       <c r="A251" t="s">
-        <v>250</v>
+        <v>246</v>
       </c>
       <c r="B251">
-        <v>641816</v>
+        <v>669422</v>
       </c>
       <c r="C251" t="s">
         <v>285</v>
@@ -3986,10 +3977,10 @@
     </row>
     <row r="252" spans="1:3">
       <c r="A252" t="s">
-        <v>251</v>
+        <v>247</v>
       </c>
       <c r="B252">
-        <v>676106</v>
+        <v>657376</v>
       </c>
       <c r="C252" t="s">
         <v>285</v>
@@ -3997,7 +3988,10 @@
     </row>
     <row r="253" spans="1:3">
       <c r="A253" t="s">
-        <v>252</v>
+        <v>248</v>
+      </c>
+      <c r="B253">
+        <v>676508</v>
       </c>
       <c r="C253" t="s">
         <v>285</v>
@@ -4005,21 +3999,21 @@
     </row>
     <row r="254" spans="1:3">
       <c r="A254" t="s">
-        <v>253</v>
+        <v>249</v>
       </c>
       <c r="B254">
-        <v>489119</v>
+        <v>687223</v>
       </c>
       <c r="C254" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
     </row>
     <row r="255" spans="1:3">
       <c r="A255" t="s">
-        <v>254</v>
+        <v>250</v>
       </c>
       <c r="B255">
-        <v>670102</v>
+        <v>656288</v>
       </c>
       <c r="C255" t="s">
         <v>285</v>
@@ -4027,7 +4021,10 @@
     </row>
     <row r="256" spans="1:3">
       <c r="A256" t="s">
-        <v>255</v>
+        <v>251</v>
+      </c>
+      <c r="B256">
+        <v>687765</v>
       </c>
       <c r="C256" t="s">
         <v>285</v>
@@ -4035,10 +4032,10 @@
     </row>
     <row r="257" spans="1:3">
       <c r="A257" t="s">
-        <v>256</v>
+        <v>252</v>
       </c>
       <c r="B257">
-        <v>656731</v>
+        <v>641816</v>
       </c>
       <c r="C257" t="s">
         <v>285</v>
@@ -4046,10 +4043,10 @@
     </row>
     <row r="258" spans="1:3">
       <c r="A258" t="s">
-        <v>257</v>
+        <v>253</v>
       </c>
       <c r="B258">
-        <v>676961</v>
+        <v>676106</v>
       </c>
       <c r="C258" t="s">
         <v>285</v>
@@ -4057,43 +4054,37 @@
     </row>
     <row r="259" spans="1:3">
       <c r="A259" t="s">
-        <v>258</v>
-      </c>
-      <c r="B259">
-        <v>677960</v>
+        <v>254</v>
       </c>
       <c r="C259" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
     </row>
     <row r="260" spans="1:3">
       <c r="A260" t="s">
-        <v>259</v>
+        <v>255</v>
       </c>
       <c r="B260">
-        <v>605452</v>
+        <v>489119</v>
       </c>
       <c r="C260" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="261" spans="1:3">
       <c r="A261" t="s">
-        <v>260</v>
+        <v>256</v>
       </c>
       <c r="B261">
-        <v>666142</v>
+        <v>670102</v>
       </c>
       <c r="C261" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
     </row>
     <row r="262" spans="1:3">
       <c r="A262" t="s">
-        <v>261</v>
-      </c>
-      <c r="B262">
-        <v>689017</v>
+        <v>257</v>
       </c>
       <c r="C262" t="s">
         <v>285</v>
@@ -4101,10 +4092,10 @@
     </row>
     <row r="263" spans="1:3">
       <c r="A263" t="s">
-        <v>262</v>
+        <v>258</v>
       </c>
       <c r="B263">
-        <v>664062</v>
+        <v>656731</v>
       </c>
       <c r="C263" t="s">
         <v>285</v>
@@ -4112,21 +4103,21 @@
     </row>
     <row r="264" spans="1:3">
       <c r="A264" t="s">
-        <v>263</v>
+        <v>259</v>
       </c>
       <c r="B264">
-        <v>676428</v>
+        <v>676961</v>
       </c>
       <c r="C264" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
     </row>
     <row r="265" spans="1:3">
       <c r="A265" t="s">
-        <v>264</v>
+        <v>260</v>
       </c>
       <c r="B265">
-        <v>676974</v>
+        <v>605452</v>
       </c>
       <c r="C265" t="s">
         <v>285</v>
@@ -4134,21 +4125,21 @@
     </row>
     <row r="266" spans="1:3">
       <c r="A266" t="s">
-        <v>265</v>
+        <v>261</v>
       </c>
       <c r="B266">
-        <v>669203</v>
+        <v>666142</v>
       </c>
       <c r="C266" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="267" spans="1:3">
       <c r="A267" t="s">
-        <v>266</v>
+        <v>262</v>
       </c>
       <c r="B267">
-        <v>680684</v>
+        <v>689017</v>
       </c>
       <c r="C267" t="s">
         <v>285</v>
@@ -4156,10 +4147,10 @@
     </row>
     <row r="268" spans="1:3">
       <c r="A268" t="s">
-        <v>267</v>
+        <v>263</v>
       </c>
       <c r="B268">
-        <v>700363</v>
+        <v>664062</v>
       </c>
       <c r="C268" t="s">
         <v>285</v>
@@ -4167,21 +4158,21 @@
     </row>
     <row r="269" spans="1:3">
       <c r="A269" t="s">
-        <v>268</v>
+        <v>264</v>
       </c>
       <c r="B269">
-        <v>663465</v>
+        <v>676428</v>
       </c>
       <c r="C269" t="s">
-        <v>284</v>
+        <v>286</v>
       </c>
     </row>
     <row r="270" spans="1:3">
       <c r="A270" t="s">
-        <v>269</v>
+        <v>265</v>
       </c>
       <c r="B270">
-        <v>695549</v>
+        <v>676974</v>
       </c>
       <c r="C270" t="s">
         <v>285</v>
@@ -4189,21 +4180,21 @@
     </row>
     <row r="271" spans="1:3">
       <c r="A271" t="s">
-        <v>270</v>
+        <v>266</v>
       </c>
       <c r="B271">
-        <v>663738</v>
+        <v>669203</v>
       </c>
       <c r="C271" t="s">
-        <v>284</v>
+        <v>285</v>
       </c>
     </row>
     <row r="272" spans="1:3">
       <c r="A272" t="s">
-        <v>271</v>
+        <v>267</v>
       </c>
       <c r="B272">
-        <v>701656</v>
+        <v>680684</v>
       </c>
       <c r="C272" t="s">
         <v>285</v>
@@ -4211,10 +4202,10 @@
     </row>
     <row r="273" spans="1:3">
       <c r="A273" t="s">
-        <v>272</v>
+        <v>268</v>
       </c>
       <c r="B273">
-        <v>694646</v>
+        <v>700363</v>
       </c>
       <c r="C273" t="s">
         <v>285</v>
@@ -4222,21 +4213,21 @@
     </row>
     <row r="274" spans="1:3">
       <c r="A274" t="s">
-        <v>273</v>
+        <v>269</v>
       </c>
       <c r="B274">
-        <v>669387</v>
+        <v>663465</v>
       </c>
       <c r="C274" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="275" spans="1:3">
       <c r="A275" t="s">
-        <v>274</v>
+        <v>270</v>
       </c>
       <c r="B275">
-        <v>502043</v>
+        <v>695549</v>
       </c>
       <c r="C275" t="s">
         <v>285</v>
@@ -4244,21 +4235,21 @@
     </row>
     <row r="276" spans="1:3">
       <c r="A276" t="s">
-        <v>275</v>
+        <v>271</v>
       </c>
       <c r="B276">
-        <v>669854</v>
+        <v>663738</v>
       </c>
       <c r="C276" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="277" spans="1:3">
       <c r="A277" t="s">
-        <v>276</v>
+        <v>272</v>
       </c>
       <c r="B277">
-        <v>668964</v>
+        <v>701656</v>
       </c>
       <c r="C277" t="s">
         <v>285</v>
@@ -4266,10 +4257,10 @@
     </row>
     <row r="278" spans="1:3">
       <c r="A278" t="s">
-        <v>277</v>
+        <v>273</v>
       </c>
       <c r="B278">
-        <v>695534</v>
+        <v>694646</v>
       </c>
       <c r="C278" t="s">
         <v>285</v>
@@ -4277,10 +4268,10 @@
     </row>
     <row r="279" spans="1:3">
       <c r="A279" t="s">
-        <v>278</v>
+        <v>274</v>
       </c>
       <c r="B279">
-        <v>663855</v>
+        <v>669387</v>
       </c>
       <c r="C279" t="s">
         <v>285</v>
@@ -4288,10 +4279,10 @@
     </row>
     <row r="280" spans="1:3">
       <c r="A280" t="s">
-        <v>279</v>
+        <v>275</v>
       </c>
       <c r="B280">
-        <v>594902</v>
+        <v>502043</v>
       </c>
       <c r="C280" t="s">
         <v>285</v>
@@ -4299,10 +4290,10 @@
     </row>
     <row r="281" spans="1:3">
       <c r="A281" t="s">
-        <v>280</v>
+        <v>276</v>
       </c>
       <c r="B281">
-        <v>656557</v>
+        <v>669854</v>
       </c>
       <c r="C281" t="s">
         <v>285</v>
@@ -4310,10 +4301,10 @@
     </row>
     <row r="282" spans="1:3">
       <c r="A282" t="s">
-        <v>281</v>
+        <v>277</v>
       </c>
       <c r="B282">
-        <v>669713</v>
+        <v>668964</v>
       </c>
       <c r="C282" t="s">
         <v>285</v>
@@ -4321,10 +4312,10 @@
     </row>
     <row r="283" spans="1:3">
       <c r="A283" t="s">
-        <v>282</v>
+        <v>278</v>
       </c>
       <c r="B283">
-        <v>663372</v>
+        <v>695534</v>
       </c>
       <c r="C283" t="s">
         <v>285</v>
@@ -4332,12 +4323,67 @@
     </row>
     <row r="284" spans="1:3">
       <c r="A284" t="s">
+        <v>279</v>
+      </c>
+      <c r="B284">
+        <v>663855</v>
+      </c>
+      <c r="C284" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="285" spans="1:3">
+      <c r="A285" t="s">
+        <v>280</v>
+      </c>
+      <c r="B285">
+        <v>594902</v>
+      </c>
+      <c r="C285" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="286" spans="1:3">
+      <c r="A286" t="s">
+        <v>281</v>
+      </c>
+      <c r="B286">
+        <v>656557</v>
+      </c>
+      <c r="C286" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="287" spans="1:3">
+      <c r="A287" t="s">
+        <v>282</v>
+      </c>
+      <c r="B287">
+        <v>669713</v>
+      </c>
+      <c r="C287" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="288" spans="1:3">
+      <c r="A288" t="s">
         <v>283</v>
       </c>
-      <c r="B284">
+      <c r="B288">
+        <v>663372</v>
+      </c>
+      <c r="C288" t="s">
+        <v>285</v>
+      </c>
+    </row>
+    <row r="289" spans="1:3">
+      <c r="A289" t="s">
+        <v>284</v>
+      </c>
+      <c r="B289">
         <v>686249</v>
       </c>
-      <c r="C284" t="s">
+      <c r="C289" t="s">
         <v>285</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Add pitcher images and update historical starters for new lineup
- Added 29 new pitcher headshot images
- Updated Historical_Starting_Pitchers.xlsx with today's starters
- Total pitcher images now: 52

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/backend/data/mlb/Historical_Starting_Pitchers.xlsx
+++ b/backend/data/mlb/Historical_Starting_Pitchers.xlsx
@@ -25,6 +25,96 @@
     <t>Handedness</t>
   </si>
   <si>
+    <t>Adrian Houser</t>
+  </si>
+  <si>
+    <t>Andrew Abbott</t>
+  </si>
+  <si>
+    <t>Cade Cavalli</t>
+  </si>
+  <si>
+    <t>Chris Sale</t>
+  </si>
+  <si>
+    <t>Cristopher Sánchez</t>
+  </si>
+  <si>
+    <t>Drew Rasmussen</t>
+  </si>
+  <si>
+    <t>Freddy Peralta</t>
+  </si>
+  <si>
+    <t>Garrett Crochet</t>
+  </si>
+  <si>
+    <t>Gavin Williams</t>
+  </si>
+  <si>
+    <t>George Kirby</t>
+  </si>
+  <si>
+    <t>Joe Ryan</t>
+  </si>
+  <si>
+    <t>Kevin Gausman</t>
+  </si>
+  <si>
+    <t>Kyle Freeland</t>
+  </si>
+  <si>
+    <t>Luis Severino</t>
+  </si>
+  <si>
+    <t>Matthew Boyd</t>
+  </si>
+  <si>
+    <t>Matthew Liberatore</t>
+  </si>
+  <si>
+    <t>Nathan Eovaldi</t>
+  </si>
+  <si>
+    <t>Nick Pivetta</t>
+  </si>
+  <si>
+    <t>Paul Skenes</t>
+  </si>
+  <si>
+    <t>Sandy Alcantara</t>
+  </si>
+  <si>
+    <t>Tarik Skubal</t>
+  </si>
+  <si>
+    <t>Trevor Rogers</t>
+  </si>
+  <si>
+    <t>Yoshinobu Yamamoto</t>
+  </si>
+  <si>
+    <t>Yusei Kikuchi</t>
+  </si>
+  <si>
+    <t>Zac Gallen</t>
+  </si>
+  <si>
+    <t>Shane Smith</t>
+  </si>
+  <si>
+    <t>Noah Cameron</t>
+  </si>
+  <si>
+    <t>Mike Burrows</t>
+  </si>
+  <si>
+    <t>Jacob Misiorowski</t>
+  </si>
+  <si>
+    <t>Cam Schlittler</t>
+  </si>
+  <si>
     <t>Bryce Elder</t>
   </si>
   <si>
@@ -97,42 +187,21 @@
     <t>Chase Burns</t>
   </si>
   <si>
-    <t>Cristopher Sánchez</t>
-  </si>
-  <si>
-    <t>Freddy Peralta</t>
-  </si>
-  <si>
-    <t>George Kirby</t>
-  </si>
-  <si>
     <t>Keider Montero</t>
   </si>
   <si>
-    <t>Kevin Gausman</t>
-  </si>
-  <si>
     <t>Luis Gil</t>
   </si>
   <si>
-    <t>Matthew Boyd</t>
-  </si>
-  <si>
     <t>Shohei Ohtani</t>
   </si>
   <si>
-    <t>Andrew Abbott</t>
-  </si>
-  <si>
     <t>Caden Dana</t>
   </si>
   <si>
     <t>Casey Mize</t>
   </si>
   <si>
-    <t>Chris Sale</t>
-  </si>
-  <si>
     <t>Dean Kremer</t>
   </si>
   <si>
@@ -157,9 +226,6 @@
     <t>José Suarez</t>
   </si>
   <si>
-    <t>Kyle Freeland</t>
-  </si>
-  <si>
     <t>Logan Gilbert</t>
   </si>
   <si>
@@ -178,9 +244,6 @@
     <t>Michael Wacha</t>
   </si>
   <si>
-    <t>Paul Skenes</t>
-  </si>
-  <si>
     <t>Ryan Pepiot</t>
   </si>
   <si>
@@ -193,15 +256,9 @@
     <t>Zebby Matthews</t>
   </si>
   <si>
-    <t>Shane Smith</t>
-  </si>
-  <si>
     <t>Cade Horton</t>
   </si>
   <si>
-    <t>Cam Schlittler</t>
-  </si>
-  <si>
     <t>Connelly Early</t>
   </si>
   <si>
@@ -223,9 +280,6 @@
     <t>Kyle Bradish</t>
   </si>
   <si>
-    <t>Matthew Liberatore</t>
-  </si>
-  <si>
     <t>Mitchell Parker</t>
   </si>
   <si>
@@ -235,9 +289,6 @@
     <t>Spencer Strider</t>
   </si>
   <si>
-    <t>Zac Gallen</t>
-  </si>
-  <si>
     <t>Zack Littell</t>
   </si>
   <si>
@@ -268,9 +319,6 @@
     <t>Colin Rea</t>
   </si>
   <si>
-    <t>Drew Rasmussen</t>
-  </si>
-  <si>
     <t>Dylan Cease</t>
   </si>
   <si>
@@ -280,9 +328,6 @@
     <t>Hunter Greene</t>
   </si>
   <si>
-    <t>Luis Severino</t>
-  </si>
-  <si>
     <t>Max Fried</t>
   </si>
   <si>
@@ -304,9 +349,6 @@
     <t>Tanner Gordon</t>
   </si>
   <si>
-    <t>Jacob Misiorowski</t>
-  </si>
-  <si>
     <t>Parker Messick</t>
   </si>
   <si>
@@ -352,9 +394,6 @@
     <t>Jesus Luzardo</t>
   </si>
   <si>
-    <t>Joe Ryan</t>
-  </si>
-  <si>
     <t>Lucas Giolito</t>
   </si>
   <si>
@@ -367,27 +406,12 @@
     <t>Randy Vásquez</t>
   </si>
   <si>
-    <t>Sandy Alcantara</t>
-  </si>
-  <si>
     <t>Shane Baz</t>
   </si>
   <si>
     <t>Tanner Bibee</t>
   </si>
   <si>
-    <t>Tarik Skubal</t>
-  </si>
-  <si>
-    <t>Trevor Rogers</t>
-  </si>
-  <si>
-    <t>Yoshinobu Yamamoto</t>
-  </si>
-  <si>
-    <t>Yusei Kikuchi</t>
-  </si>
-  <si>
     <t>Brad Lord</t>
   </si>
   <si>
@@ -403,9 +427,6 @@
     <t>David Peterson</t>
   </si>
   <si>
-    <t>Gavin Williams</t>
-  </si>
-  <si>
     <t>Jack Flaherty</t>
   </si>
   <si>
@@ -418,9 +439,6 @@
     <t>José Soriano</t>
   </si>
   <si>
-    <t>Nick Pivetta</t>
-  </si>
-  <si>
     <t>Pablo López</t>
   </si>
   <si>
@@ -466,15 +484,9 @@
     <t>Taj Bradley</t>
   </si>
   <si>
-    <t>Noah Cameron</t>
-  </si>
-  <si>
     <t>Aaron Nola</t>
   </si>
   <si>
-    <t>Adrian Houser</t>
-  </si>
-  <si>
     <t>Cade Povich</t>
   </si>
   <si>
@@ -508,12 +520,6 @@
     <t>Bryan Woo</t>
   </si>
   <si>
-    <t>Cade Cavalli</t>
-  </si>
-  <si>
-    <t>Garrett Crochet</t>
-  </si>
-  <si>
     <t>Joey Wentz</t>
   </si>
   <si>
@@ -616,9 +622,6 @@
     <t>Mick Abel</t>
   </si>
   <si>
-    <t>Mike Burrows</t>
-  </si>
-  <si>
     <t>Victor Mederos</t>
   </si>
   <si>
@@ -641,9 +644,6 @@
   </si>
   <si>
     <t>Erick Fedde</t>
-  </si>
-  <si>
-    <t>Nathan Eovaldi</t>
   </si>
   <si>
     <t>Carlos Carrasco</t>
@@ -1251,7 +1251,7 @@
         <v>3</v>
       </c>
       <c r="B2">
-        <v>693821</v>
+        <v>605288</v>
       </c>
       <c r="C2" t="s">
         <v>285</v>
@@ -1262,10 +1262,10 @@
         <v>4</v>
       </c>
       <c r="B3">
-        <v>605135</v>
+        <v>671096</v>
       </c>
       <c r="C3" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="4" spans="1:3">
@@ -1273,7 +1273,7 @@
         <v>5</v>
       </c>
       <c r="B4">
-        <v>663978</v>
+        <v>676917</v>
       </c>
       <c r="C4" t="s">
         <v>285</v>
@@ -1284,23 +1284,29 @@
         <v>6</v>
       </c>
       <c r="B5">
-        <v>605280</v>
+        <v>519242</v>
       </c>
       <c r="C5" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="6" spans="1:3">
+      <c r="A6" t="s">
+        <v>7</v>
+      </c>
+      <c r="B6">
+        <v>650911</v>
+      </c>
       <c r="C6" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="7" spans="1:3">
       <c r="A7" t="s">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B7">
-        <v>663436</v>
+        <v>656876</v>
       </c>
       <c r="C7" t="s">
         <v>285</v>
@@ -1308,18 +1314,21 @@
     </row>
     <row r="8" spans="1:3">
       <c r="A8" t="s">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B8">
-        <v>665795</v>
+        <v>642547</v>
       </c>
       <c r="C8" t="s">
         <v>285</v>
       </c>
     </row>
     <row r="9" spans="1:3">
+      <c r="A9" t="s">
+        <v>10</v>
+      </c>
       <c r="B9">
-        <v>656492</v>
+        <v>676979</v>
       </c>
       <c r="C9" t="s">
         <v>286</v>
@@ -1327,10 +1336,10 @@
     </row>
     <row r="10" spans="1:3">
       <c r="A10" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="B10">
-        <v>683004</v>
+        <v>668909</v>
       </c>
       <c r="C10" t="s">
         <v>285</v>
@@ -1338,10 +1347,10 @@
     </row>
     <row r="11" spans="1:3">
       <c r="A11" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B11">
-        <v>434378</v>
+        <v>669923</v>
       </c>
       <c r="C11" t="s">
         <v>285</v>
@@ -1349,43 +1358,43 @@
     </row>
     <row r="12" spans="1:3">
       <c r="A12" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="B12">
-        <v>663460</v>
+        <v>657746</v>
       </c>
       <c r="C12" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="13" spans="1:3">
       <c r="A13" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B13">
-        <v>690986</v>
+        <v>592332</v>
       </c>
       <c r="C13" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="14" spans="1:3">
       <c r="A14" t="s">
-        <v>13</v>
+        <v>15</v>
       </c>
       <c r="B14">
-        <v>689017</v>
+        <v>607536</v>
       </c>
       <c r="C14" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="15" spans="1:3">
       <c r="A15" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B15">
-        <v>622491</v>
+        <v>622663</v>
       </c>
       <c r="C15" t="s">
         <v>285</v>
@@ -1393,54 +1402,54 @@
     </row>
     <row r="16" spans="1:3">
       <c r="A16" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B16">
-        <v>647336</v>
+        <v>571510</v>
       </c>
       <c r="C16" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="17" spans="1:3">
       <c r="A17" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="B17">
-        <v>607259</v>
+        <v>669461</v>
       </c>
       <c r="C17" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="18" spans="1:3">
       <c r="A18" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="B18">
-        <v>624133</v>
+        <v>543135</v>
       </c>
       <c r="C18" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="19" spans="1:3">
       <c r="A19" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="B19">
-        <v>677960</v>
+        <v>601713</v>
       </c>
       <c r="C19" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="20" spans="1:3">
       <c r="A20" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="B20">
-        <v>680573</v>
+        <v>694973</v>
       </c>
       <c r="C20" t="s">
         <v>285</v>
@@ -1448,10 +1457,10 @@
     </row>
     <row r="21" spans="1:3">
       <c r="A21" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="B21">
-        <v>592836</v>
+        <v>645261</v>
       </c>
       <c r="C21" t="s">
         <v>285</v>
@@ -1459,32 +1468,32 @@
     </row>
     <row r="22" spans="1:3">
       <c r="A22" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="B22">
-        <v>621111</v>
+        <v>669373</v>
       </c>
       <c r="C22" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="23" spans="1:3">
       <c r="A23" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
       <c r="B23">
-        <v>808963</v>
+        <v>669432</v>
       </c>
       <c r="C23" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="24" spans="1:3">
       <c r="A24" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="B24">
-        <v>608372</v>
+        <v>808967</v>
       </c>
       <c r="C24" t="s">
         <v>285</v>
@@ -1492,10 +1501,10 @@
     </row>
     <row r="25" spans="1:3">
       <c r="A25" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="B25">
-        <v>682052</v>
+        <v>579328</v>
       </c>
       <c r="C25" t="s">
         <v>286</v>
@@ -1503,10 +1512,10 @@
     </row>
     <row r="26" spans="1:3">
       <c r="A26" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="B26">
-        <v>677952</v>
+        <v>668678</v>
       </c>
       <c r="C26" t="s">
         <v>285</v>
@@ -1514,56 +1523,65 @@
     </row>
     <row r="27" spans="1:3">
       <c r="A27" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="B27">
-        <v>695505</v>
+        <v>681343</v>
       </c>
       <c r="C27" t="s">
         <v>285</v>
       </c>
     </row>
     <row r="28" spans="1:3">
+      <c r="A28" t="s">
+        <v>29</v>
+      </c>
       <c r="B28">
-        <v>696270</v>
+        <v>702070</v>
       </c>
       <c r="C28" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="29" spans="1:3">
+      <c r="A29" t="s">
+        <v>30</v>
+      </c>
       <c r="B29">
-        <v>681517</v>
+        <v>681347</v>
       </c>
       <c r="C29" t="s">
         <v>285</v>
       </c>
     </row>
     <row r="30" spans="1:3">
+      <c r="A30" t="s">
+        <v>31</v>
+      </c>
       <c r="B30">
-        <v>800048</v>
+        <v>694819</v>
       </c>
       <c r="C30" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="31" spans="1:3">
       <c r="A31" t="s">
-        <v>27</v>
+        <v>32</v>
       </c>
       <c r="B31">
-        <v>650911</v>
+        <v>693645</v>
       </c>
       <c r="C31" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="32" spans="1:3">
       <c r="A32" t="s">
-        <v>28</v>
+        <v>33</v>
       </c>
       <c r="B32">
-        <v>642547</v>
+        <v>693821</v>
       </c>
       <c r="C32" t="s">
         <v>285</v>
@@ -1571,10 +1589,10 @@
     </row>
     <row r="33" spans="1:3">
       <c r="A33" t="s">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="B33">
-        <v>669923</v>
+        <v>605135</v>
       </c>
       <c r="C33" t="s">
         <v>285</v>
@@ -1582,10 +1600,10 @@
     </row>
     <row r="34" spans="1:3">
       <c r="A34" t="s">
-        <v>30</v>
+        <v>35</v>
       </c>
       <c r="B34">
-        <v>672456</v>
+        <v>663978</v>
       </c>
       <c r="C34" t="s">
         <v>285</v>
@@ -1593,54 +1611,45 @@
     </row>
     <row r="35" spans="1:3">
       <c r="A35" t="s">
-        <v>31</v>
+        <v>36</v>
       </c>
       <c r="B35">
-        <v>592332</v>
+        <v>605280</v>
       </c>
       <c r="C35" t="s">
         <v>285</v>
       </c>
     </row>
     <row r="36" spans="1:3">
-      <c r="A36" t="s">
-        <v>32</v>
-      </c>
-      <c r="B36">
-        <v>661563</v>
-      </c>
       <c r="C36" t="s">
         <v>285</v>
       </c>
     </row>
     <row r="37" spans="1:3">
       <c r="A37" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="B37">
-        <v>571510</v>
+        <v>663436</v>
       </c>
       <c r="C37" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="38" spans="1:3">
       <c r="A38" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="B38">
-        <v>660271</v>
+        <v>665795</v>
       </c>
       <c r="C38" t="s">
         <v>285</v>
       </c>
     </row>
     <row r="39" spans="1:3">
-      <c r="A39" t="s">
-        <v>35</v>
-      </c>
       <c r="B39">
-        <v>671096</v>
+        <v>656492</v>
       </c>
       <c r="C39" t="s">
         <v>286</v>
@@ -1648,10 +1657,10 @@
     </row>
     <row r="40" spans="1:3">
       <c r="A40" t="s">
-        <v>36</v>
+        <v>39</v>
       </c>
       <c r="B40">
-        <v>702674</v>
+        <v>683004</v>
       </c>
       <c r="C40" t="s">
         <v>285</v>
@@ -1659,10 +1668,10 @@
     </row>
     <row r="41" spans="1:3">
       <c r="A41" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="B41">
-        <v>663554</v>
+        <v>434378</v>
       </c>
       <c r="C41" t="s">
         <v>285</v>
@@ -1670,10 +1679,10 @@
     </row>
     <row r="42" spans="1:3">
       <c r="A42" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="B42">
-        <v>519242</v>
+        <v>663460</v>
       </c>
       <c r="C42" t="s">
         <v>286</v>
@@ -1681,32 +1690,32 @@
     </row>
     <row r="43" spans="1:3">
       <c r="A43" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="B43">
-        <v>665152</v>
+        <v>690986</v>
       </c>
       <c r="C43" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="44" spans="1:3">
       <c r="A44" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="B44">
-        <v>593958</v>
+        <v>689017</v>
       </c>
       <c r="C44" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="45" spans="1:3">
       <c r="A45" t="s">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="B45">
-        <v>691587</v>
+        <v>622491</v>
       </c>
       <c r="C45" t="s">
         <v>285</v>
@@ -1714,10 +1723,10 @@
     </row>
     <row r="46" spans="1:3">
       <c r="A46" t="s">
-        <v>42</v>
+        <v>45</v>
       </c>
       <c r="B46">
-        <v>663623</v>
+        <v>647336</v>
       </c>
       <c r="C46" t="s">
         <v>285</v>
@@ -1725,21 +1734,21 @@
     </row>
     <row r="47" spans="1:3">
       <c r="A47" t="s">
-        <v>43</v>
+        <v>46</v>
       </c>
       <c r="B47">
-        <v>605488</v>
+        <v>607259</v>
       </c>
       <c r="C47" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="48" spans="1:3">
       <c r="A48" t="s">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="B48">
-        <v>676282</v>
+        <v>624133</v>
       </c>
       <c r="C48" t="s">
         <v>286</v>
@@ -1747,43 +1756,43 @@
     </row>
     <row r="49" spans="1:3">
       <c r="A49" t="s">
-        <v>45</v>
+        <v>48</v>
       </c>
       <c r="B49">
-        <v>621244</v>
+        <v>677960</v>
       </c>
       <c r="C49" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="50" spans="1:3">
       <c r="A50" t="s">
-        <v>46</v>
+        <v>49</v>
       </c>
       <c r="B50">
-        <v>660761</v>
+        <v>680573</v>
       </c>
       <c r="C50" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="51" spans="1:3">
       <c r="A51" t="s">
-        <v>47</v>
+        <v>50</v>
       </c>
       <c r="B51">
-        <v>607536</v>
+        <v>592836</v>
       </c>
       <c r="C51" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="52" spans="1:3">
       <c r="A52" t="s">
-        <v>48</v>
+        <v>51</v>
       </c>
       <c r="B52">
-        <v>669302</v>
+        <v>621111</v>
       </c>
       <c r="C52" t="s">
         <v>285</v>
@@ -1791,21 +1800,21 @@
     </row>
     <row r="53" spans="1:3">
       <c r="A53" t="s">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="B53">
-        <v>669022</v>
+        <v>808963</v>
       </c>
       <c r="C53" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="54" spans="1:3">
       <c r="A54" t="s">
-        <v>50</v>
+        <v>53</v>
       </c>
       <c r="B54">
-        <v>518876</v>
+        <v>608372</v>
       </c>
       <c r="C54" t="s">
         <v>285</v>
@@ -1813,21 +1822,21 @@
     </row>
     <row r="55" spans="1:3">
       <c r="A55" t="s">
-        <v>51</v>
+        <v>54</v>
       </c>
       <c r="B55">
-        <v>650633</v>
+        <v>682052</v>
       </c>
       <c r="C55" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="56" spans="1:3">
       <c r="A56" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="B56">
-        <v>700241</v>
+        <v>677952</v>
       </c>
       <c r="C56" t="s">
         <v>285</v>
@@ -1835,43 +1844,34 @@
     </row>
     <row r="57" spans="1:3">
       <c r="A57" t="s">
-        <v>53</v>
+        <v>56</v>
       </c>
       <c r="B57">
-        <v>608379</v>
+        <v>695505</v>
       </c>
       <c r="C57" t="s">
         <v>285</v>
       </c>
     </row>
     <row r="58" spans="1:3">
-      <c r="A58" t="s">
-        <v>54</v>
-      </c>
       <c r="B58">
-        <v>694973</v>
+        <v>696270</v>
       </c>
       <c r="C58" t="s">
         <v>285</v>
       </c>
     </row>
     <row r="59" spans="1:3">
-      <c r="A59" t="s">
-        <v>55</v>
-      </c>
       <c r="B59">
-        <v>686752</v>
+        <v>681517</v>
       </c>
       <c r="C59" t="s">
         <v>285</v>
       </c>
     </row>
     <row r="60" spans="1:3">
-      <c r="A60" t="s">
-        <v>56</v>
-      </c>
       <c r="B60">
-        <v>640455</v>
+        <v>800048</v>
       </c>
       <c r="C60" t="s">
         <v>286</v>
@@ -1882,7 +1882,7 @@
         <v>57</v>
       </c>
       <c r="B61">
-        <v>663941</v>
+        <v>672456</v>
       </c>
       <c r="C61" t="s">
         <v>285</v>
@@ -1893,7 +1893,7 @@
         <v>58</v>
       </c>
       <c r="B62">
-        <v>805673</v>
+        <v>661563</v>
       </c>
       <c r="C62" t="s">
         <v>285</v>
@@ -1904,7 +1904,7 @@
         <v>59</v>
       </c>
       <c r="B63">
-        <v>681343</v>
+        <v>660271</v>
       </c>
       <c r="C63" t="s">
         <v>285</v>
@@ -1915,7 +1915,7 @@
         <v>60</v>
       </c>
       <c r="B64">
-        <v>690990</v>
+        <v>702674</v>
       </c>
       <c r="C64" t="s">
         <v>285</v>
@@ -1926,7 +1926,7 @@
         <v>61</v>
       </c>
       <c r="B65">
-        <v>693645</v>
+        <v>663554</v>
       </c>
       <c r="C65" t="s">
         <v>285</v>
@@ -1937,10 +1937,10 @@
         <v>62</v>
       </c>
       <c r="B66">
-        <v>813349</v>
+        <v>665152</v>
       </c>
       <c r="C66" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="67" spans="1:3">
@@ -1948,10 +1948,10 @@
         <v>63</v>
       </c>
       <c r="B67">
-        <v>805123</v>
+        <v>593958</v>
       </c>
       <c r="C67" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="68" spans="1:3">
@@ -1959,10 +1959,10 @@
         <v>64</v>
       </c>
       <c r="B68">
-        <v>607074</v>
+        <v>691587</v>
       </c>
       <c r="C68" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="69" spans="1:3">
@@ -1970,7 +1970,7 @@
         <v>65</v>
       </c>
       <c r="B69">
-        <v>686218</v>
+        <v>663623</v>
       </c>
       <c r="C69" t="s">
         <v>285</v>
@@ -1981,10 +1981,10 @@
         <v>66</v>
       </c>
       <c r="B70">
-        <v>592791</v>
+        <v>605488</v>
       </c>
       <c r="C70" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="71" spans="1:3">
@@ -1992,10 +1992,10 @@
         <v>67</v>
       </c>
       <c r="B71">
-        <v>671212</v>
+        <v>676282</v>
       </c>
       <c r="C71" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="72" spans="1:3">
@@ -2003,7 +2003,7 @@
         <v>68</v>
       </c>
       <c r="B72">
-        <v>680694</v>
+        <v>621244</v>
       </c>
       <c r="C72" t="s">
         <v>285</v>
@@ -2014,7 +2014,7 @@
         <v>69</v>
       </c>
       <c r="B73">
-        <v>669461</v>
+        <v>660761</v>
       </c>
       <c r="C73" t="s">
         <v>286</v>
@@ -2025,10 +2025,10 @@
         <v>70</v>
       </c>
       <c r="B74">
-        <v>680730</v>
+        <v>669302</v>
       </c>
       <c r="C74" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="75" spans="1:3">
@@ -2036,10 +2036,10 @@
         <v>71</v>
       </c>
       <c r="B75">
-        <v>680732</v>
+        <v>669022</v>
       </c>
       <c r="C75" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="76" spans="1:3">
@@ -2047,7 +2047,7 @@
         <v>72</v>
       </c>
       <c r="B76">
-        <v>675911</v>
+        <v>518876</v>
       </c>
       <c r="C76" t="s">
         <v>285</v>
@@ -2058,7 +2058,7 @@
         <v>73</v>
       </c>
       <c r="B77">
-        <v>668678</v>
+        <v>650633</v>
       </c>
       <c r="C77" t="s">
         <v>285</v>
@@ -2069,7 +2069,7 @@
         <v>74</v>
       </c>
       <c r="B78">
-        <v>641793</v>
+        <v>700241</v>
       </c>
       <c r="C78" t="s">
         <v>285</v>
@@ -2080,7 +2080,7 @@
         <v>75</v>
       </c>
       <c r="B79">
-        <v>669920</v>
+        <v>608379</v>
       </c>
       <c r="C79" t="s">
         <v>285</v>
@@ -2091,7 +2091,7 @@
         <v>76</v>
       </c>
       <c r="B80">
-        <v>678906</v>
+        <v>686752</v>
       </c>
       <c r="C80" t="s">
         <v>285</v>
@@ -2102,10 +2102,10 @@
         <v>77</v>
       </c>
       <c r="B81">
-        <v>702056</v>
+        <v>640455</v>
       </c>
       <c r="C81" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="82" spans="1:3">
@@ -2113,7 +2113,7 @@
         <v>78</v>
       </c>
       <c r="B82">
-        <v>800049</v>
+        <v>663941</v>
       </c>
       <c r="C82" t="s">
         <v>285</v>
@@ -2124,7 +2124,7 @@
         <v>79</v>
       </c>
       <c r="B83">
-        <v>641927</v>
+        <v>805673</v>
       </c>
       <c r="C83" t="s">
         <v>285</v>
@@ -2135,7 +2135,7 @@
         <v>80</v>
       </c>
       <c r="B84">
-        <v>678394</v>
+        <v>690990</v>
       </c>
       <c r="C84" t="s">
         <v>285</v>
@@ -2146,10 +2146,10 @@
         <v>81</v>
       </c>
       <c r="B85">
-        <v>450203</v>
+        <v>813349</v>
       </c>
       <c r="C85" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="86" spans="1:3">
@@ -2157,10 +2157,10 @@
         <v>82</v>
       </c>
       <c r="B86">
-        <v>477132</v>
+        <v>805123</v>
       </c>
       <c r="C86" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="87" spans="1:3">
@@ -2168,10 +2168,10 @@
         <v>83</v>
       </c>
       <c r="B87">
-        <v>607067</v>
+        <v>607074</v>
       </c>
       <c r="C87" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="88" spans="1:3">
@@ -2179,7 +2179,7 @@
         <v>84</v>
       </c>
       <c r="B88">
-        <v>656876</v>
+        <v>686218</v>
       </c>
       <c r="C88" t="s">
         <v>285</v>
@@ -2190,7 +2190,7 @@
         <v>85</v>
       </c>
       <c r="B89">
-        <v>656302</v>
+        <v>592791</v>
       </c>
       <c r="C89" t="s">
         <v>285</v>
@@ -2201,10 +2201,10 @@
         <v>86</v>
       </c>
       <c r="B90">
-        <v>664285</v>
+        <v>671212</v>
       </c>
       <c r="C90" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="91" spans="1:3">
@@ -2212,7 +2212,7 @@
         <v>87</v>
       </c>
       <c r="B91">
-        <v>668881</v>
+        <v>680694</v>
       </c>
       <c r="C91" t="s">
         <v>285</v>
@@ -2223,10 +2223,10 @@
         <v>88</v>
       </c>
       <c r="B92">
-        <v>622663</v>
+        <v>680730</v>
       </c>
       <c r="C92" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="93" spans="1:3">
@@ -2234,10 +2234,10 @@
         <v>89</v>
       </c>
       <c r="B93">
-        <v>608331</v>
+        <v>680732</v>
       </c>
       <c r="C93" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="94" spans="1:3">
@@ -2245,7 +2245,7 @@
         <v>90</v>
       </c>
       <c r="B94">
-        <v>453286</v>
+        <v>675911</v>
       </c>
       <c r="C94" t="s">
         <v>285</v>
@@ -2256,7 +2256,7 @@
         <v>91</v>
       </c>
       <c r="B95">
-        <v>547179</v>
+        <v>641793</v>
       </c>
       <c r="C95" t="s">
         <v>285</v>
@@ -2267,10 +2267,10 @@
         <v>92</v>
       </c>
       <c r="B96">
-        <v>571578</v>
+        <v>669920</v>
       </c>
       <c r="C96" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="97" spans="1:3">
@@ -2278,7 +2278,7 @@
         <v>93</v>
       </c>
       <c r="B97">
-        <v>669194</v>
+        <v>678906</v>
       </c>
       <c r="C97" t="s">
         <v>285</v>
@@ -2289,7 +2289,7 @@
         <v>94</v>
       </c>
       <c r="B98">
-        <v>543243</v>
+        <v>702056</v>
       </c>
       <c r="C98" t="s">
         <v>285</v>
@@ -2300,7 +2300,7 @@
         <v>95</v>
       </c>
       <c r="B99">
-        <v>685299</v>
+        <v>800049</v>
       </c>
       <c r="C99" t="s">
         <v>285</v>
@@ -2311,7 +2311,7 @@
         <v>96</v>
       </c>
       <c r="B100">
-        <v>694819</v>
+        <v>641927</v>
       </c>
       <c r="C100" t="s">
         <v>285</v>
@@ -2322,10 +2322,10 @@
         <v>97</v>
       </c>
       <c r="B101">
-        <v>800048</v>
+        <v>678394</v>
       </c>
       <c r="C101" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="102" spans="1:3">
@@ -2333,7 +2333,7 @@
         <v>98</v>
       </c>
       <c r="B102">
-        <v>696149</v>
+        <v>450203</v>
       </c>
       <c r="C102" t="s">
         <v>285</v>
@@ -2344,7 +2344,7 @@
         <v>99</v>
       </c>
       <c r="B103">
-        <v>674841</v>
+        <v>477132</v>
       </c>
       <c r="C103" t="s">
         <v>286</v>
@@ -2355,10 +2355,10 @@
         <v>100</v>
       </c>
       <c r="B104">
-        <v>815083</v>
+        <v>607067</v>
       </c>
       <c r="C104" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="105" spans="1:3">
@@ -2366,7 +2366,7 @@
         <v>101</v>
       </c>
       <c r="B105">
-        <v>687075</v>
+        <v>656302</v>
       </c>
       <c r="C105" t="s">
         <v>285</v>
@@ -2377,10 +2377,10 @@
         <v>102</v>
       </c>
       <c r="B106">
-        <v>669467</v>
+        <v>664285</v>
       </c>
       <c r="C106" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="107" spans="1:3">
@@ -2388,7 +2388,7 @@
         <v>103</v>
       </c>
       <c r="B107">
-        <v>663903</v>
+        <v>668881</v>
       </c>
       <c r="C107" t="s">
         <v>285</v>
@@ -2399,10 +2399,10 @@
         <v>104</v>
       </c>
       <c r="B108">
-        <v>694297</v>
+        <v>608331</v>
       </c>
       <c r="C108" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="109" spans="1:3">
@@ -2410,7 +2410,7 @@
         <v>105</v>
       </c>
       <c r="B109">
-        <v>605540</v>
+        <v>453286</v>
       </c>
       <c r="C109" t="s">
         <v>285</v>
@@ -2421,7 +2421,7 @@
         <v>106</v>
       </c>
       <c r="B110">
-        <v>682243</v>
+        <v>547179</v>
       </c>
       <c r="C110" t="s">
         <v>285</v>
@@ -2432,10 +2432,10 @@
         <v>107</v>
       </c>
       <c r="B111">
-        <v>686613</v>
+        <v>571578</v>
       </c>
       <c r="C111" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="112" spans="1:3">
@@ -2443,7 +2443,7 @@
         <v>108</v>
       </c>
       <c r="B112">
-        <v>694462</v>
+        <v>669194</v>
       </c>
       <c r="C112" t="s">
         <v>285</v>
@@ -2454,7 +2454,7 @@
         <v>109</v>
       </c>
       <c r="B113">
-        <v>669372</v>
+        <v>543243</v>
       </c>
       <c r="C113" t="s">
         <v>285</v>
@@ -2465,7 +2465,7 @@
         <v>110</v>
       </c>
       <c r="B114">
-        <v>594798</v>
+        <v>685299</v>
       </c>
       <c r="C114" t="s">
         <v>285</v>
@@ -2476,7 +2476,7 @@
         <v>111</v>
       </c>
       <c r="B115">
-        <v>666200</v>
+        <v>800048</v>
       </c>
       <c r="C115" t="s">
         <v>286</v>
@@ -2487,7 +2487,7 @@
         <v>112</v>
       </c>
       <c r="B116">
-        <v>657746</v>
+        <v>696149</v>
       </c>
       <c r="C116" t="s">
         <v>285</v>
@@ -2498,10 +2498,10 @@
         <v>113</v>
       </c>
       <c r="B117">
-        <v>608337</v>
+        <v>674841</v>
       </c>
       <c r="C117" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="118" spans="1:3">
@@ -2509,7 +2509,7 @@
         <v>114</v>
       </c>
       <c r="B118">
-        <v>527048</v>
+        <v>815083</v>
       </c>
       <c r="C118" t="s">
         <v>286</v>
@@ -2520,7 +2520,7 @@
         <v>115</v>
       </c>
       <c r="B119">
-        <v>656605</v>
+        <v>687075</v>
       </c>
       <c r="C119" t="s">
         <v>285</v>
@@ -2531,7 +2531,7 @@
         <v>116</v>
       </c>
       <c r="B120">
-        <v>681190</v>
+        <v>669467</v>
       </c>
       <c r="C120" t="s">
         <v>285</v>
@@ -2542,7 +2542,7 @@
         <v>117</v>
       </c>
       <c r="B121">
-        <v>645261</v>
+        <v>663903</v>
       </c>
       <c r="C121" t="s">
         <v>285</v>
@@ -2553,7 +2553,7 @@
         <v>118</v>
       </c>
       <c r="B122">
-        <v>669358</v>
+        <v>694297</v>
       </c>
       <c r="C122" t="s">
         <v>285</v>
@@ -2564,7 +2564,7 @@
         <v>119</v>
       </c>
       <c r="B123">
-        <v>676440</v>
+        <v>605540</v>
       </c>
       <c r="C123" t="s">
         <v>285</v>
@@ -2575,10 +2575,10 @@
         <v>120</v>
       </c>
       <c r="B124">
-        <v>669373</v>
+        <v>682243</v>
       </c>
       <c r="C124" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="125" spans="1:3">
@@ -2586,10 +2586,10 @@
         <v>121</v>
       </c>
       <c r="B125">
-        <v>669432</v>
+        <v>686613</v>
       </c>
       <c r="C125" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="126" spans="1:3">
@@ -2597,7 +2597,7 @@
         <v>122</v>
       </c>
       <c r="B126">
-        <v>808967</v>
+        <v>694462</v>
       </c>
       <c r="C126" t="s">
         <v>285</v>
@@ -2608,10 +2608,10 @@
         <v>123</v>
       </c>
       <c r="B127">
-        <v>579328</v>
+        <v>669372</v>
       </c>
       <c r="C127" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="128" spans="1:3">
@@ -2619,7 +2619,7 @@
         <v>124</v>
       </c>
       <c r="B128">
-        <v>695418</v>
+        <v>594798</v>
       </c>
       <c r="C128" t="s">
         <v>285</v>
@@ -2630,10 +2630,10 @@
         <v>125</v>
       </c>
       <c r="B129">
-        <v>663568</v>
+        <v>666200</v>
       </c>
       <c r="C129" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="130" spans="1:3">
@@ -2641,7 +2641,7 @@
         <v>126</v>
       </c>
       <c r="B130">
-        <v>685326</v>
+        <v>608337</v>
       </c>
       <c r="C130" t="s">
         <v>285</v>
@@ -2652,10 +2652,10 @@
         <v>127</v>
       </c>
       <c r="B131">
-        <v>804636</v>
+        <v>527048</v>
       </c>
       <c r="C131" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="132" spans="1:3">
@@ -2663,10 +2663,10 @@
         <v>128</v>
       </c>
       <c r="B132">
-        <v>656849</v>
+        <v>656605</v>
       </c>
       <c r="C132" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="133" spans="1:3">
@@ -2674,7 +2674,7 @@
         <v>129</v>
       </c>
       <c r="B133">
-        <v>668909</v>
+        <v>681190</v>
       </c>
       <c r="C133" t="s">
         <v>285</v>
@@ -2685,7 +2685,7 @@
         <v>130</v>
       </c>
       <c r="B134">
-        <v>656427</v>
+        <v>669358</v>
       </c>
       <c r="C134" t="s">
         <v>285</v>
@@ -2696,7 +2696,7 @@
         <v>131</v>
       </c>
       <c r="B135">
-        <v>665871</v>
+        <v>676440</v>
       </c>
       <c r="C135" t="s">
         <v>285</v>
@@ -2707,7 +2707,7 @@
         <v>132</v>
       </c>
       <c r="B136">
-        <v>670912</v>
+        <v>695418</v>
       </c>
       <c r="C136" t="s">
         <v>285</v>
@@ -2718,7 +2718,7 @@
         <v>133</v>
       </c>
       <c r="B137">
-        <v>667755</v>
+        <v>663568</v>
       </c>
       <c r="C137" t="s">
         <v>285</v>
@@ -2729,7 +2729,7 @@
         <v>134</v>
       </c>
       <c r="B138">
-        <v>601713</v>
+        <v>685326</v>
       </c>
       <c r="C138" t="s">
         <v>285</v>
@@ -2740,7 +2740,7 @@
         <v>135</v>
       </c>
       <c r="B139">
-        <v>641154</v>
+        <v>804636</v>
       </c>
       <c r="C139" t="s">
         <v>285</v>
@@ -2751,10 +2751,10 @@
         <v>136</v>
       </c>
       <c r="B140">
-        <v>682990</v>
+        <v>656849</v>
       </c>
       <c r="C140" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="141" spans="1:3">
@@ -2762,7 +2762,7 @@
         <v>137</v>
       </c>
       <c r="B141">
-        <v>678368</v>
+        <v>656427</v>
       </c>
       <c r="C141" t="s">
         <v>285</v>
@@ -2773,10 +2773,10 @@
         <v>138</v>
       </c>
       <c r="B142">
-        <v>676467</v>
+        <v>665871</v>
       </c>
       <c r="C142" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="143" spans="1:3">
@@ -2784,7 +2784,7 @@
         <v>139</v>
       </c>
       <c r="B143">
-        <v>693313</v>
+        <v>670912</v>
       </c>
       <c r="C143" t="s">
         <v>285</v>
@@ -2795,10 +2795,10 @@
         <v>140</v>
       </c>
       <c r="B144">
-        <v>693855</v>
+        <v>667755</v>
       </c>
       <c r="C144" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="145" spans="1:3">
@@ -2806,10 +2806,10 @@
         <v>141</v>
       </c>
       <c r="B145">
-        <v>801139</v>
+        <v>641154</v>
       </c>
       <c r="C145" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="146" spans="1:3">
@@ -2817,7 +2817,7 @@
         <v>142</v>
       </c>
       <c r="B146">
-        <v>686930</v>
+        <v>682990</v>
       </c>
       <c r="C146" t="s">
         <v>285</v>
@@ -2828,7 +2828,7 @@
         <v>143</v>
       </c>
       <c r="B147">
-        <v>607192</v>
+        <v>678368</v>
       </c>
       <c r="C147" t="s">
         <v>285</v>
@@ -2839,7 +2839,7 @@
         <v>144</v>
       </c>
       <c r="B148">
-        <v>605483</v>
+        <v>676467</v>
       </c>
       <c r="C148" t="s">
         <v>286</v>
@@ -2850,7 +2850,7 @@
         <v>145</v>
       </c>
       <c r="B149">
-        <v>664299</v>
+        <v>693313</v>
       </c>
       <c r="C149" t="s">
         <v>285</v>
@@ -2861,10 +2861,10 @@
         <v>146</v>
       </c>
       <c r="B150">
-        <v>686563</v>
+        <v>693855</v>
       </c>
       <c r="C150" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="151" spans="1:3">
@@ -2872,10 +2872,10 @@
         <v>147</v>
       </c>
       <c r="B151">
-        <v>543294</v>
+        <v>801139</v>
       </c>
       <c r="C151" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="152" spans="1:3">
@@ -2883,10 +2883,10 @@
         <v>148</v>
       </c>
       <c r="B152">
-        <v>671106</v>
+        <v>686930</v>
       </c>
       <c r="C152" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="153" spans="1:3">
@@ -2894,7 +2894,7 @@
         <v>149</v>
       </c>
       <c r="B153">
-        <v>671737</v>
+        <v>607192</v>
       </c>
       <c r="C153" t="s">
         <v>285</v>
@@ -2905,7 +2905,7 @@
         <v>150</v>
       </c>
       <c r="B154">
-        <v>702070</v>
+        <v>605483</v>
       </c>
       <c r="C154" t="s">
         <v>286</v>
@@ -2916,7 +2916,7 @@
         <v>151</v>
       </c>
       <c r="B155">
-        <v>605400</v>
+        <v>664299</v>
       </c>
       <c r="C155" t="s">
         <v>285</v>
@@ -2927,7 +2927,7 @@
         <v>152</v>
       </c>
       <c r="B156">
-        <v>605288</v>
+        <v>686563</v>
       </c>
       <c r="C156" t="s">
         <v>285</v>
@@ -2938,10 +2938,10 @@
         <v>153</v>
       </c>
       <c r="B157">
-        <v>700249</v>
+        <v>543294</v>
       </c>
       <c r="C157" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="158" spans="1:3">
@@ -2949,10 +2949,10 @@
         <v>154</v>
       </c>
       <c r="B158">
-        <v>669160</v>
+        <v>671106</v>
       </c>
       <c r="C158" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="159" spans="1:3">
@@ -2960,7 +2960,7 @@
         <v>155</v>
       </c>
       <c r="B159">
-        <v>608566</v>
+        <v>671737</v>
       </c>
       <c r="C159" t="s">
         <v>285</v>
@@ -2971,10 +2971,10 @@
         <v>156</v>
       </c>
       <c r="B160">
-        <v>500779</v>
+        <v>605400</v>
       </c>
       <c r="C160" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="161" spans="1:3">
@@ -2982,7 +2982,7 @@
         <v>157</v>
       </c>
       <c r="B161">
-        <v>641482</v>
+        <v>700249</v>
       </c>
       <c r="C161" t="s">
         <v>286</v>
@@ -2993,10 +2993,10 @@
         <v>158</v>
       </c>
       <c r="B162">
-        <v>592662</v>
+        <v>669160</v>
       </c>
       <c r="C162" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="163" spans="1:3">
@@ -3004,7 +3004,7 @@
         <v>159</v>
       </c>
       <c r="B163">
-        <v>669456</v>
+        <v>608566</v>
       </c>
       <c r="C163" t="s">
         <v>285</v>
@@ -3015,10 +3015,10 @@
         <v>160</v>
       </c>
       <c r="B164">
-        <v>701542</v>
+        <v>500779</v>
       </c>
       <c r="C164" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="165" spans="1:3">
@@ -3026,10 +3026,10 @@
         <v>161</v>
       </c>
       <c r="B165">
-        <v>686701</v>
+        <v>641482</v>
       </c>
       <c r="C165" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="166" spans="1:3">
@@ -3037,10 +3037,10 @@
         <v>162</v>
       </c>
       <c r="B166">
-        <v>672782</v>
+        <v>592662</v>
       </c>
       <c r="C166" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="167" spans="1:3">
@@ -3048,7 +3048,7 @@
         <v>163</v>
       </c>
       <c r="B167">
-        <v>693433</v>
+        <v>669456</v>
       </c>
       <c r="C167" t="s">
         <v>285</v>
@@ -3059,7 +3059,7 @@
         <v>164</v>
       </c>
       <c r="B168">
-        <v>676917</v>
+        <v>701542</v>
       </c>
       <c r="C168" t="s">
         <v>285</v>
@@ -3070,10 +3070,10 @@
         <v>165</v>
       </c>
       <c r="B169">
-        <v>676979</v>
+        <v>686701</v>
       </c>
       <c r="C169" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="170" spans="1:3">
@@ -3081,10 +3081,10 @@
         <v>166</v>
       </c>
       <c r="B170">
-        <v>666214</v>
+        <v>672782</v>
       </c>
       <c r="C170" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="171" spans="1:3">
@@ -3092,7 +3092,7 @@
         <v>167</v>
       </c>
       <c r="B171">
-        <v>657277</v>
+        <v>693433</v>
       </c>
       <c r="C171" t="s">
         <v>285</v>
@@ -3103,10 +3103,10 @@
         <v>168</v>
       </c>
       <c r="B172">
-        <v>571945</v>
+        <v>666214</v>
       </c>
       <c r="C172" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="173" spans="1:3">
@@ -3114,7 +3114,7 @@
         <v>169</v>
       </c>
       <c r="B173">
-        <v>622503</v>
+        <v>657277</v>
       </c>
       <c r="C173" t="s">
         <v>285</v>
@@ -3125,10 +3125,10 @@
         <v>170</v>
       </c>
       <c r="B174">
-        <v>666157</v>
+        <v>571945</v>
       </c>
       <c r="C174" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="175" spans="1:3">
@@ -3136,10 +3136,10 @@
         <v>171</v>
       </c>
       <c r="B175">
-        <v>684007</v>
+        <v>622503</v>
       </c>
       <c r="C175" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="176" spans="1:3">
@@ -3147,10 +3147,10 @@
         <v>172</v>
       </c>
       <c r="B176">
-        <v>677944</v>
+        <v>666157</v>
       </c>
       <c r="C176" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="177" spans="1:3">
@@ -3158,10 +3158,10 @@
         <v>173</v>
       </c>
       <c r="B177">
-        <v>669330</v>
+        <v>684007</v>
       </c>
       <c r="C177" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="178" spans="1:3">
@@ -3169,7 +3169,7 @@
         <v>174</v>
       </c>
       <c r="B178">
-        <v>506433</v>
+        <v>677944</v>
       </c>
       <c r="C178" t="s">
         <v>285</v>
@@ -3180,7 +3180,7 @@
         <v>175</v>
       </c>
       <c r="B179">
-        <v>687830</v>
+        <v>669330</v>
       </c>
       <c r="C179" t="s">
         <v>285</v>
@@ -3191,10 +3191,10 @@
         <v>176</v>
       </c>
       <c r="B180">
-        <v>656641</v>
+        <v>506433</v>
       </c>
       <c r="C180" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="181" spans="1:3">
@@ -3202,7 +3202,7 @@
         <v>177</v>
       </c>
       <c r="B181">
-        <v>690997</v>
+        <v>687830</v>
       </c>
       <c r="C181" t="s">
         <v>285</v>
@@ -3213,10 +3213,10 @@
         <v>178</v>
       </c>
       <c r="B182">
-        <v>669060</v>
+        <v>656641</v>
       </c>
       <c r="C182" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="183" spans="1:3">
@@ -3224,7 +3224,7 @@
         <v>179</v>
       </c>
       <c r="B183">
-        <v>801403</v>
+        <v>690997</v>
       </c>
       <c r="C183" t="s">
         <v>285</v>
@@ -3235,7 +3235,7 @@
         <v>180</v>
       </c>
       <c r="B184">
-        <v>806960</v>
+        <v>669060</v>
       </c>
       <c r="C184" t="s">
         <v>285</v>
@@ -3246,7 +3246,7 @@
         <v>181</v>
       </c>
       <c r="B185">
-        <v>678215</v>
+        <v>801403</v>
       </c>
       <c r="C185" t="s">
         <v>285</v>
@@ -3257,7 +3257,7 @@
         <v>182</v>
       </c>
       <c r="B186">
-        <v>673540</v>
+        <v>806960</v>
       </c>
       <c r="C186" t="s">
         <v>285</v>
@@ -3268,10 +3268,10 @@
         <v>183</v>
       </c>
       <c r="B187">
-        <v>606996</v>
+        <v>678215</v>
       </c>
       <c r="C187" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="188" spans="1:3">
@@ -3279,7 +3279,7 @@
         <v>184</v>
       </c>
       <c r="B188">
-        <v>681293</v>
+        <v>673540</v>
       </c>
       <c r="C188" t="s">
         <v>285</v>
@@ -3290,10 +3290,10 @@
         <v>185</v>
       </c>
       <c r="B189">
-        <v>607625</v>
+        <v>606996</v>
       </c>
       <c r="C189" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="190" spans="1:3">
@@ -3301,10 +3301,10 @@
         <v>186</v>
       </c>
       <c r="B190">
-        <v>542881</v>
+        <v>681293</v>
       </c>
       <c r="C190" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="191" spans="1:3">
@@ -3312,7 +3312,7 @@
         <v>187</v>
       </c>
       <c r="B191">
-        <v>615698</v>
+        <v>607625</v>
       </c>
       <c r="C191" t="s">
         <v>285</v>
@@ -3323,10 +3323,10 @@
         <v>188</v>
       </c>
       <c r="B192">
-        <v>650644</v>
+        <v>542881</v>
       </c>
       <c r="C192" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="193" spans="1:3">
@@ -3334,10 +3334,10 @@
         <v>189</v>
       </c>
       <c r="B193">
-        <v>687931</v>
+        <v>615698</v>
       </c>
       <c r="C193" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="194" spans="1:3">
@@ -3345,10 +3345,10 @@
         <v>190</v>
       </c>
       <c r="B194">
-        <v>641778</v>
+        <v>650644</v>
       </c>
       <c r="C194" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="195" spans="1:3">
@@ -3356,10 +3356,10 @@
         <v>191</v>
       </c>
       <c r="B195">
-        <v>686799</v>
+        <v>687931</v>
       </c>
       <c r="C195" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="196" spans="1:3">
@@ -3367,10 +3367,10 @@
         <v>192</v>
       </c>
       <c r="B196">
-        <v>672710</v>
+        <v>641778</v>
       </c>
       <c r="C196" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="197" spans="1:3">
@@ -3378,7 +3378,7 @@
         <v>193</v>
       </c>
       <c r="B197">
-        <v>687473</v>
+        <v>686799</v>
       </c>
       <c r="C197" t="s">
         <v>285</v>
@@ -3389,7 +3389,7 @@
         <v>194</v>
       </c>
       <c r="B198">
-        <v>674370</v>
+        <v>672710</v>
       </c>
       <c r="C198" t="s">
         <v>285</v>
@@ -3400,10 +3400,10 @@
         <v>195</v>
       </c>
       <c r="B199">
-        <v>676664</v>
+        <v>687473</v>
       </c>
       <c r="C199" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="200" spans="1:3">
@@ -3411,7 +3411,7 @@
         <v>196</v>
       </c>
       <c r="B200">
-        <v>690916</v>
+        <v>674370</v>
       </c>
       <c r="C200" t="s">
         <v>285</v>
@@ -3422,7 +3422,7 @@
         <v>197</v>
       </c>
       <c r="B201">
-        <v>688107</v>
+        <v>676664</v>
       </c>
       <c r="C201" t="s">
         <v>286</v>
@@ -3433,7 +3433,7 @@
         <v>198</v>
       </c>
       <c r="B202">
-        <v>676083</v>
+        <v>690916</v>
       </c>
       <c r="C202" t="s">
         <v>285</v>
@@ -3444,10 +3444,10 @@
         <v>199</v>
       </c>
       <c r="B203">
-        <v>690953</v>
+        <v>688107</v>
       </c>
       <c r="C203" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="204" spans="1:3">
@@ -3455,7 +3455,7 @@
         <v>200</v>
       </c>
       <c r="B204">
-        <v>681347</v>
+        <v>676083</v>
       </c>
       <c r="C204" t="s">
         <v>285</v>
@@ -3466,7 +3466,7 @@
         <v>201</v>
       </c>
       <c r="B205">
-        <v>682929</v>
+        <v>690953</v>
       </c>
       <c r="C205" t="s">
         <v>285</v>
@@ -3477,7 +3477,7 @@
         <v>202</v>
       </c>
       <c r="B206">
-        <v>570632</v>
+        <v>682929</v>
       </c>
       <c r="C206" t="s">
         <v>285</v>
@@ -3488,7 +3488,7 @@
         <v>203</v>
       </c>
       <c r="B207">
-        <v>687064</v>
+        <v>570632</v>
       </c>
       <c r="C207" t="s">
         <v>285</v>
@@ -3499,7 +3499,7 @@
         <v>204</v>
       </c>
       <c r="B208">
-        <v>678022</v>
+        <v>687064</v>
       </c>
       <c r="C208" t="s">
         <v>285</v>
@@ -3510,26 +3510,26 @@
         <v>205</v>
       </c>
       <c r="B209">
-        <v>596295</v>
+        <v>678022</v>
       </c>
       <c r="C209" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="210" spans="1:3">
       <c r="A210" t="s">
-        <v>65</v>
+        <v>206</v>
+      </c>
+      <c r="B210">
+        <v>596295</v>
       </c>
       <c r="C210" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="211" spans="1:3">
       <c r="A211" t="s">
-        <v>206</v>
-      </c>
-      <c r="B211">
-        <v>694477</v>
+        <v>84</v>
       </c>
       <c r="C211" t="s">
         <v>285</v>
@@ -3540,10 +3540,10 @@
         <v>207</v>
       </c>
       <c r="B212">
-        <v>571760</v>
+        <v>694477</v>
       </c>
       <c r="C212" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="213" spans="1:3">
@@ -3551,10 +3551,10 @@
         <v>208</v>
       </c>
       <c r="B213">
-        <v>607200</v>
+        <v>571760</v>
       </c>
       <c r="C213" t="s">
-        <v>285</v>
+        <v>286</v>
       </c>
     </row>
     <row r="214" spans="1:3">
@@ -3562,7 +3562,7 @@
         <v>209</v>
       </c>
       <c r="B214">
-        <v>543135</v>
+        <v>607200</v>
       </c>
       <c r="C214" t="s">
         <v>285</v>

</xml_diff>